<commit_message>
Update panel C data again (73 genes, adds detoxification module)
Panel C now uses the latest mecA+ACME workbook, extending the
flanking region further downstream with a new "Putative
detoxification module" (10 modules total, up from 9).
</commit_message>
<xml_diff>
--- a/figures/shap_heatmaps/data/JE2_mecA_ACME.xlsx
+++ b/figures/shap_heatmaps/data/JE2_mecA_ACME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/paultorrillo/Downloads/hunting_for_good_shaps/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{F18A7198-252A-D74A-91CD-BE087BF706FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{7CAEEF9F-33FC-B946-8072-76C542BB5523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-160" yWindow="-19360" windowWidth="27240" windowHeight="15440"/>
+    <workbookView xWindow="1920" yWindow="2120" windowWidth="26040" windowHeight="13940"/>
   </bookViews>
   <sheets>
     <sheet name="selected_gene_directional_shap" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="160">
   <si>
     <t>row_gene_idx</t>
   </si>
@@ -226,6 +226,27 @@
     <t>col_1047:FEOBHI_12070 NADPH-dependent 2,4-dienoyl-CoA reductase, sulfur reductase, or a related oxidoreductase</t>
   </si>
   <si>
+    <t>col_1570:FEOBHI_12075 putative tRNA-dihydrouridine synthase</t>
+  </si>
+  <si>
+    <t>col_283:FEOBHI_12080 TfoX N-terminal domain protein</t>
+  </si>
+  <si>
+    <t>col_1848:FEOBHI_12085 MFS domain-containing protein</t>
+  </si>
+  <si>
+    <t>col_682:FEOBHI_12090 Flavodoxin</t>
+  </si>
+  <si>
+    <t>col_1357:FEOBHI_12095 HTH-type transcriptional regulator GltR</t>
+  </si>
+  <si>
+    <t>col_769:FEOBHI_12100 DUF4865 domain-containing protein</t>
+  </si>
+  <si>
+    <t>col_1141:FEOBHI_12105 HTH-type transcriptional regulator YofA</t>
+  </si>
+  <si>
     <t>FEOBHI_09970 response regulator YycF</t>
   </si>
   <si>
@@ -427,13 +448,28 @@
     <t>FEOBHI_12070 NADPH-dependent 2,4-dienoyl-CoA reductase, sulfur reductase, or a related oxidoreductase</t>
   </si>
   <si>
-    <t>Group</t>
+    <t>FEOBHI_12075 putative tRNA-dihydrouridine synthase</t>
   </si>
   <si>
-    <t>sulfide response</t>
+    <t>FEOBHI_12080 TfoX N-terminal domain protein</t>
   </si>
   <si>
-    <t>sulfide response (split sqr gene)</t>
+    <t>FEOBHI_12085 MFS domain-containing protein</t>
+  </si>
+  <si>
+    <t>FEOBHI_12090 Flavodoxin</t>
+  </si>
+  <si>
+    <t>FEOBHI_12095 HTH-type transcriptional regulator GltR</t>
+  </si>
+  <si>
+    <t>FEOBHI_12100 DUF4865 domain-containing protein</t>
+  </si>
+  <si>
+    <t>FEOBHI_12105 HTH-type transcriptional regulator YofA</t>
+  </si>
+  <si>
+    <t>Group</t>
   </si>
   <si>
     <t>cell wall homeostasis</t>
@@ -455,6 +491,15 @@
   </si>
   <si>
     <t>copper resistance (ACME)</t>
+  </si>
+  <si>
+    <t>sulfide response</t>
+  </si>
+  <si>
+    <t>sulfide response (split sqr gene)</t>
+  </si>
+  <si>
+    <t>Putative detoxification module</t>
   </si>
 </sst>
 </file>
@@ -1296,19 +1341,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BQ67"/>
+  <dimension ref="A1:BX74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="21.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="90.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="C1" t="s">
         <v>1</v>
@@ -1511,19 +1556,40 @@
       <c r="BQ1" t="s">
         <v>67</v>
       </c>
+      <c r="BR1" t="s">
+        <v>68</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>69</v>
+      </c>
+      <c r="BT1" t="s">
+        <v>70</v>
+      </c>
+      <c r="BU1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BV1" t="s">
+        <v>72</v>
+      </c>
+      <c r="BW1" t="s">
+        <v>73</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>74</v>
+      </c>
     </row>
-    <row r="2" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>1075</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D2" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="E2" s="1">
         <v>8.1999999999999994E-6</v>
@@ -1720,22 +1786,43 @@
       <c r="BQ2" s="1">
         <v>-2.5700000000000001E-5</v>
       </c>
+      <c r="BR2" s="1">
+        <v>3.6900000000000002E-5</v>
+      </c>
+      <c r="BS2" s="1">
+        <v>-1.5999999999999999E-5</v>
+      </c>
+      <c r="BT2" s="1">
+        <v>-1.2300000000000001E-5</v>
+      </c>
+      <c r="BU2" s="1">
+        <v>-2.1399999999999998E-5</v>
+      </c>
+      <c r="BV2" s="1">
+        <v>-2.1399999999999998E-5</v>
+      </c>
+      <c r="BW2" s="1">
+        <v>-1.8700000000000001E-5</v>
+      </c>
+      <c r="BX2" s="1">
+        <v>-2.0800000000000001E-5</v>
+      </c>
     </row>
-    <row r="3" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>2197</v>
       </c>
       <c r="B3" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D3" s="1">
         <v>3.2400000000000001E-5</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="F3" s="1">
         <v>2.8600000000000001E-5</v>
@@ -1929,16 +2016,37 @@
       <c r="BQ3" s="1">
         <v>-1.8700000000000001E-5</v>
       </c>
+      <c r="BR3" s="1">
+        <v>2.7699999999999999E-5</v>
+      </c>
+      <c r="BS3" s="1">
+        <v>-5.9000000000000003E-6</v>
+      </c>
+      <c r="BT3" s="1">
+        <v>4.4799999999999998E-5</v>
+      </c>
+      <c r="BU3" s="1">
+        <v>-1.66E-5</v>
+      </c>
+      <c r="BV3" s="1">
+        <v>2.6800000000000001E-5</v>
+      </c>
+      <c r="BW3" s="1">
+        <v>-4.6E-6</v>
+      </c>
+      <c r="BX3" s="1">
+        <v>-1.5099999999999999E-5</v>
+      </c>
     </row>
-    <row r="4" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>1947</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D4">
         <v>1.3125999999999999E-3</v>
@@ -1947,7 +2055,7 @@
         <v>1.2105E-3</v>
       </c>
       <c r="F4" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="G4">
         <v>6.4999999999999997E-4</v>
@@ -2138,16 +2246,37 @@
       <c r="BQ4">
         <v>-1.0965E-3</v>
       </c>
+      <c r="BR4">
+        <v>1.3772999999999999E-3</v>
+      </c>
+      <c r="BS4">
+        <v>-8.6830000000000002E-4</v>
+      </c>
+      <c r="BT4">
+        <v>1.9900000000000001E-4</v>
+      </c>
+      <c r="BU4">
+        <v>-9.3849999999999999E-4</v>
+      </c>
+      <c r="BV4">
+        <v>-4.2860000000000001E-4</v>
+      </c>
+      <c r="BW4">
+        <v>-8.34E-4</v>
+      </c>
+      <c r="BX4">
+        <v>-8.5680000000000001E-4</v>
+      </c>
     </row>
-    <row r="5" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>1232</v>
       </c>
       <c r="B5" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D5">
         <v>1.41082E-2</v>
@@ -2159,7 +2288,7 @@
         <v>2.4248E-3</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="H5">
         <v>6.4879999999999998E-3</v>
@@ -2347,16 +2476,37 @@
       <c r="BQ5">
         <v>-4.7245999999999998E-3</v>
       </c>
+      <c r="BR5">
+        <v>-1.9246999999999999E-3</v>
+      </c>
+      <c r="BS5">
+        <v>1.6901300000000001E-2</v>
+      </c>
+      <c r="BT5">
+        <v>0.1391223</v>
+      </c>
+      <c r="BU5">
+        <v>2.039E-3</v>
+      </c>
+      <c r="BV5">
+        <v>0.20133380000000001</v>
+      </c>
+      <c r="BW5">
+        <v>-1.49616E-2</v>
+      </c>
+      <c r="BX5">
+        <v>6.04127E-2</v>
+      </c>
     </row>
-    <row r="6" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>1254</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C6" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1">
         <v>4.6E-6</v>
@@ -2371,7 +2521,7 @@
         <v>1.1000000000000001E-6</v>
       </c>
       <c r="H6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="I6" s="1">
         <v>4.0999999999999997E-6</v>
@@ -2556,13 +2706,34 @@
       <c r="BQ6" s="1">
         <v>-3.5999999999999998E-6</v>
       </c>
+      <c r="BR6" s="1">
+        <v>4.6E-6</v>
+      </c>
+      <c r="BS6" s="1">
+        <v>-1.9999999999999999E-6</v>
+      </c>
+      <c r="BT6" s="1">
+        <v>-7.9999999999999996E-7</v>
+      </c>
+      <c r="BU6" s="1">
+        <v>-2.5000000000000002E-6</v>
+      </c>
+      <c r="BV6" s="1">
+        <v>-2.5000000000000002E-6</v>
+      </c>
+      <c r="BW6" s="1">
+        <v>-2.3E-6</v>
+      </c>
+      <c r="BX6" s="1">
+        <v>-2.3999999999999999E-6</v>
+      </c>
     </row>
-    <row r="7" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>2271</v>
       </c>
       <c r="C7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D7">
         <v>9.8070999999999992E-3</v>
@@ -2580,7 +2751,7 @@
         <v>1.02224E-2</v>
       </c>
       <c r="I7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="J7">
         <v>1.6829299999999998E-2</v>
@@ -2762,13 +2933,34 @@
       <c r="BQ7">
         <v>-1.9106100000000001E-2</v>
       </c>
+      <c r="BR7">
+        <v>2.8606099999999999E-2</v>
+      </c>
+      <c r="BS7">
+        <v>8.4702000000000006E-3</v>
+      </c>
+      <c r="BT7">
+        <v>-2.6078799999999999E-2</v>
+      </c>
+      <c r="BU7">
+        <v>-1.1342700000000001E-2</v>
+      </c>
+      <c r="BV7">
+        <v>4.3647600000000002E-2</v>
+      </c>
+      <c r="BW7">
+        <v>4.7899499999999998E-2</v>
+      </c>
+      <c r="BX7">
+        <v>4.0765099999999999E-2</v>
+      </c>
     </row>
-    <row r="8" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>667</v>
       </c>
       <c r="C8" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D8">
         <v>1.4276E-3</v>
@@ -2789,7 +2981,7 @@
         <v>1.1938999999999999E-3</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="K8">
         <v>-4.2039999999999997E-4</v>
@@ -2968,13 +3160,34 @@
       <c r="BQ8">
         <v>-1.1915000000000001E-3</v>
       </c>
+      <c r="BR8">
+        <v>1.5045E-3</v>
+      </c>
+      <c r="BS8">
+        <v>-9.2869999999999997E-4</v>
+      </c>
+      <c r="BT8">
+        <v>1.8320000000000001E-4</v>
+      </c>
+      <c r="BU8">
+        <v>-1.0131999999999999E-3</v>
+      </c>
+      <c r="BV8">
+        <v>-4.4519999999999998E-4</v>
+      </c>
+      <c r="BW8">
+        <v>-8.8219999999999998E-4</v>
+      </c>
+      <c r="BX8">
+        <v>-9.2009999999999998E-4</v>
+      </c>
     </row>
-    <row r="9" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>1878</v>
       </c>
       <c r="C9" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D9">
         <v>-2.2926000000000001E-3</v>
@@ -2998,7 +3211,7 @@
         <v>-5.1844999999999999E-3</v>
       </c>
       <c r="K9" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="L9">
         <v>0.41351680000000002</v>
@@ -3174,13 +3387,34 @@
       <c r="BQ9">
         <v>3.3127E-3</v>
       </c>
+      <c r="BR9">
+        <v>1.09242E-2</v>
+      </c>
+      <c r="BS9">
+        <v>1.3522899999999999E-2</v>
+      </c>
+      <c r="BT9">
+        <v>6.6462999999999994E-2</v>
+      </c>
+      <c r="BU9">
+        <v>1.24277E-2</v>
+      </c>
+      <c r="BV9">
+        <v>-5.1234000000000002E-3</v>
+      </c>
+      <c r="BW9">
+        <v>-5.4775400000000002E-2</v>
+      </c>
+      <c r="BX9">
+        <v>-1.9381700000000002E-2</v>
+      </c>
     </row>
-    <row r="10" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>1014</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D10">
         <v>-6.2830000000000004E-4</v>
@@ -3207,7 +3441,7 @@
         <v>-1.93229E-2</v>
       </c>
       <c r="L10" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="M10">
         <v>2.8211E-3</v>
@@ -3380,16 +3614,37 @@
       <c r="BQ10">
         <v>7.2895E-3</v>
       </c>
+      <c r="BR10">
+        <v>2.5900099999999999E-2</v>
+      </c>
+      <c r="BS10">
+        <v>8.6390000000000008E-3</v>
+      </c>
+      <c r="BT10">
+        <v>1.2826499999999999E-2</v>
+      </c>
+      <c r="BU10">
+        <v>-2.5300000000000002E-4</v>
+      </c>
+      <c r="BV10">
+        <v>-0.12788859999999999</v>
+      </c>
+      <c r="BW10">
+        <v>-4.6208899999999997E-2</v>
+      </c>
+      <c r="BX10">
+        <v>-2.0272600000000002E-2</v>
+      </c>
     </row>
-    <row r="11" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>46</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C11" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D11">
         <v>5.4797999999999999E-3</v>
@@ -3419,7 +3674,7 @@
         <v>0.15866130000000001</v>
       </c>
       <c r="M11" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="N11">
         <v>-0.47119759999999999</v>
@@ -3589,16 +3844,37 @@
       <c r="BQ11">
         <v>1.8435000000000001E-3</v>
       </c>
+      <c r="BR11">
+        <v>-1.7845400000000001E-2</v>
+      </c>
+      <c r="BS11">
+        <v>4.4852E-3</v>
+      </c>
+      <c r="BT11">
+        <v>2.60051E-2</v>
+      </c>
+      <c r="BU11">
+        <v>-2.1182000000000002E-3</v>
+      </c>
+      <c r="BV11">
+        <v>2.05878E-2</v>
+      </c>
+      <c r="BW11">
+        <v>-2.8377900000000001E-2</v>
+      </c>
+      <c r="BX11">
+        <v>-2.2501899999999998E-2</v>
+      </c>
     </row>
-    <row r="12" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>1159</v>
       </c>
       <c r="B12" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C12" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D12">
         <v>3.3549999999999999E-3</v>
@@ -3631,7 +3907,7 @@
         <v>-0.31142360000000002</v>
       </c>
       <c r="N12" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="O12">
         <v>-0.71049280000000004</v>
@@ -3798,16 +4074,37 @@
       <c r="BQ12">
         <v>-4.2262999999999997E-3</v>
       </c>
+      <c r="BR12">
+        <v>1.2884400000000001E-2</v>
+      </c>
+      <c r="BS12">
+        <v>5.3274000000000004E-3</v>
+      </c>
+      <c r="BT12">
+        <v>5.1471200000000002E-2</v>
+      </c>
+      <c r="BU12">
+        <v>-1.774E-3</v>
+      </c>
+      <c r="BV12">
+        <v>5.6771000000000002E-2</v>
+      </c>
+      <c r="BW12">
+        <v>-1.49988E-2</v>
+      </c>
+      <c r="BX12">
+        <v>3.0661899999999999E-2</v>
+      </c>
     </row>
-    <row r="13" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>559</v>
       </c>
       <c r="B13" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C13" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D13">
         <v>6.7690000000000003E-4</v>
@@ -3843,7 +4140,7 @@
         <v>-0.87783199999999995</v>
       </c>
       <c r="O13" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="P13">
         <v>-0.82408840000000005</v>
@@ -4007,16 +4304,37 @@
       <c r="BQ13">
         <v>-8.7516E-3</v>
       </c>
+      <c r="BR13">
+        <v>9.8291999999999997E-3</v>
+      </c>
+      <c r="BS13">
+        <v>-2.6483000000000001E-3</v>
+      </c>
+      <c r="BT13">
+        <v>3.62923E-2</v>
+      </c>
+      <c r="BU13">
+        <v>-1.0536E-3</v>
+      </c>
+      <c r="BV13">
+        <v>1.7758599999999999E-2</v>
+      </c>
+      <c r="BW13">
+        <v>-1.0839000000000001E-3</v>
+      </c>
+      <c r="BX13">
+        <v>1.5844199999999999E-2</v>
+      </c>
     </row>
-    <row r="14" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>2239</v>
       </c>
       <c r="B14" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D14">
         <v>6.0867999999999998E-3</v>
@@ -4055,7 +4373,7 @@
         <v>-0.63160159999999999</v>
       </c>
       <c r="P14" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="Q14">
         <v>2.7323099999999999E-2</v>
@@ -4216,13 +4534,34 @@
       <c r="BQ14">
         <v>-5.2785999999999996E-3</v>
       </c>
+      <c r="BR14">
+        <v>1.9107300000000001E-2</v>
+      </c>
+      <c r="BS14">
+        <v>6.4513000000000001E-3</v>
+      </c>
+      <c r="BT14">
+        <v>6.0645999999999999E-3</v>
+      </c>
+      <c r="BU14">
+        <v>1.0447E-3</v>
+      </c>
+      <c r="BV14">
+        <v>-4.3547999999999998E-3</v>
+      </c>
+      <c r="BW14">
+        <v>1.6766999999999999E-3</v>
+      </c>
+      <c r="BX14">
+        <v>1.2163800000000001E-2</v>
+      </c>
     </row>
-    <row r="15" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2355</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D15">
         <v>1.1885000000000001E-3</v>
@@ -4264,7 +4603,7 @@
         <v>0.20796190000000001</v>
       </c>
       <c r="Q15" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="R15">
         <v>0.41190399999999999</v>
@@ -4422,13 +4761,34 @@
       <c r="BQ15">
         <v>3.9443999999999998E-3</v>
       </c>
+      <c r="BR15">
+        <v>-5.9100000000000005E-4</v>
+      </c>
+      <c r="BS15">
+        <v>1.9953100000000001E-2</v>
+      </c>
+      <c r="BT15">
+        <v>3.1360600000000002E-2</v>
+      </c>
+      <c r="BU15">
+        <v>-7.3001000000000003E-3</v>
+      </c>
+      <c r="BV15">
+        <v>2.78664E-2</v>
+      </c>
+      <c r="BW15">
+        <v>6.3219700000000004E-2</v>
+      </c>
+      <c r="BX15">
+        <v>5.5714600000000003E-2</v>
+      </c>
     </row>
-    <row r="16" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>2090</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D16">
         <v>5.9870000000000001E-3</v>
@@ -4473,7 +4833,7 @@
         <v>-0.35499259999999999</v>
       </c>
       <c r="R16" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="S16">
         <v>-0.34882600000000002</v>
@@ -4628,13 +4988,34 @@
       <c r="BQ16">
         <v>2.1580200000000001E-2</v>
       </c>
+      <c r="BR16">
+        <v>-7.51251E-2</v>
+      </c>
+      <c r="BS16">
+        <v>-1.01958E-2</v>
+      </c>
+      <c r="BT16">
+        <v>-1.2168200000000001E-2</v>
+      </c>
+      <c r="BU16">
+        <v>-2.7167899999999998E-2</v>
+      </c>
+      <c r="BV16">
+        <v>-8.8428800000000002E-2</v>
+      </c>
+      <c r="BW16">
+        <v>-5.3858799999999998E-2</v>
+      </c>
+      <c r="BX16">
+        <v>-1.6970900000000001E-2</v>
+      </c>
     </row>
-    <row r="17" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>4097</v>
       </c>
       <c r="C17" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D17">
         <v>5.7711000000000004E-3</v>
@@ -4682,7 +5063,7 @@
         <v>0.1874304</v>
       </c>
       <c r="S17" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="T17">
         <v>0.1430815</v>
@@ -4834,13 +5215,34 @@
       <c r="BQ17">
         <v>-2.6149499999999999E-2</v>
       </c>
+      <c r="BR17">
+        <v>2.5564099999999999E-2</v>
+      </c>
+      <c r="BS17">
+        <v>3.6985999999999998E-3</v>
+      </c>
+      <c r="BT17">
+        <v>2.2742600000000002E-2</v>
+      </c>
+      <c r="BU17">
+        <v>4.7479000000000002E-3</v>
+      </c>
+      <c r="BV17">
+        <v>2.7342999999999998E-3</v>
+      </c>
+      <c r="BW17">
+        <v>3.7112899999999997E-2</v>
+      </c>
+      <c r="BX17">
+        <v>6.4388399999999998E-2</v>
+      </c>
     </row>
-    <row r="18" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>313</v>
       </c>
       <c r="C18" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D18">
         <v>-3.4865999999999999E-3</v>
@@ -4891,7 +5293,7 @@
         <v>-0.39887909999999999</v>
       </c>
       <c r="T18" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="U18">
         <v>-0.65070019999999995</v>
@@ -5040,13 +5442,34 @@
       <c r="BQ18">
         <v>4.6043999999999998E-3</v>
       </c>
+      <c r="BR18">
+        <v>6.1405300000000003E-2</v>
+      </c>
+      <c r="BS18">
+        <v>1.0789099999999999E-2</v>
+      </c>
+      <c r="BT18">
+        <v>1.12262E-2</v>
+      </c>
+      <c r="BU18">
+        <v>3.4638200000000001E-2</v>
+      </c>
+      <c r="BV18">
+        <v>-3.2701599999999997E-2</v>
+      </c>
+      <c r="BW18">
+        <v>5.5418500000000002E-2</v>
+      </c>
+      <c r="BX18">
+        <v>8.4603999999999999E-3</v>
+      </c>
     </row>
-    <row r="19" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>3</v>
       </c>
       <c r="C19" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D19">
         <v>-6.1744E-3</v>
@@ -5100,7 +5523,7 @@
         <v>0.28231289999999998</v>
       </c>
       <c r="U19" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="V19">
         <v>-0.3173318</v>
@@ -5246,13 +5669,34 @@
       <c r="BQ19">
         <v>2.34229E-2</v>
       </c>
+      <c r="BR19">
+        <v>2.14022E-2</v>
+      </c>
+      <c r="BS19">
+        <v>1.1738699999999999E-2</v>
+      </c>
+      <c r="BT19">
+        <v>-1.1779700000000001E-2</v>
+      </c>
+      <c r="BU19">
+        <v>3.24763E-2</v>
+      </c>
+      <c r="BV19">
+        <v>-2.6246800000000001E-2</v>
+      </c>
+      <c r="BW19">
+        <v>3.7122700000000002E-2</v>
+      </c>
+      <c r="BX19">
+        <v>4.0793000000000003E-2</v>
+      </c>
     </row>
-    <row r="20" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>393</v>
       </c>
       <c r="C20" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D20">
         <v>-6.2047999999999999E-3</v>
@@ -5309,7 +5753,7 @@
         <v>-9.7061900000000007E-2</v>
       </c>
       <c r="V20" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="W20">
         <v>0.37295970000000001</v>
@@ -5452,16 +5896,37 @@
       <c r="BQ20">
         <v>2.2022699999999999E-2</v>
       </c>
+      <c r="BR20">
+        <v>3.0223799999999999E-2</v>
+      </c>
+      <c r="BS20">
+        <v>5.0746999999999997E-3</v>
+      </c>
+      <c r="BT20">
+        <v>-3.1889199999999999E-2</v>
+      </c>
+      <c r="BU20">
+        <v>3.4412199999999997E-2</v>
+      </c>
+      <c r="BV20">
+        <v>-1.6216299999999999E-2</v>
+      </c>
+      <c r="BW20">
+        <v>7.6591300000000001E-2</v>
+      </c>
+      <c r="BX20">
+        <v>5.4493699999999999E-2</v>
+      </c>
     </row>
-    <row r="21" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2620</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D21">
         <v>6.0559000000000003E-3</v>
@@ -5521,7 +5986,7 @@
         <v>-0.3184613</v>
       </c>
       <c r="W21" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="X21">
         <v>-0.84253120000000004</v>
@@ -5661,16 +6126,37 @@
       <c r="BQ21">
         <v>-4.7637000000000001E-3</v>
       </c>
+      <c r="BR21">
+        <v>-6.6455899999999998E-2</v>
+      </c>
+      <c r="BS21">
+        <v>1.0528E-3</v>
+      </c>
+      <c r="BT21">
+        <v>4.7923000000000002E-3</v>
+      </c>
+      <c r="BU21">
+        <v>2.0174399999999999E-2</v>
+      </c>
+      <c r="BV21">
+        <v>1.8466000000000001E-3</v>
+      </c>
+      <c r="BW21">
+        <v>-1.07329E-2</v>
+      </c>
+      <c r="BX21">
+        <v>-4.3170699999999999E-2</v>
+      </c>
     </row>
-    <row r="22" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2591</v>
       </c>
       <c r="B22" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C22" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D22">
         <v>3.4956000000000002E-3</v>
@@ -5733,7 +6219,7 @@
         <v>-0.50008370000000002</v>
       </c>
       <c r="X22" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="Y22">
         <v>-0.26681379999999999</v>
@@ -5870,16 +6356,37 @@
       <c r="BQ22">
         <v>-1.6490899999999999E-2</v>
       </c>
+      <c r="BR22">
+        <v>-8.0943000000000005E-3</v>
+      </c>
+      <c r="BS22">
+        <v>-3.7182000000000001E-3</v>
+      </c>
+      <c r="BT22">
+        <v>-4.9868799999999998E-2</v>
+      </c>
+      <c r="BU22">
+        <v>2.9713099999999999E-2</v>
+      </c>
+      <c r="BV22">
+        <v>-3.90876E-2</v>
+      </c>
+      <c r="BW22">
+        <v>-2.43518E-2</v>
+      </c>
+      <c r="BX22">
+        <v>-2.14751E-2</v>
+      </c>
     </row>
-    <row r="23" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2188</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D23">
         <v>2.2472999999999998E-3</v>
@@ -5945,7 +6452,7 @@
         <v>-0.30767990000000001</v>
       </c>
       <c r="Y23" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="Z23">
         <v>-0.17026230000000001</v>
@@ -6079,16 +6586,37 @@
       <c r="BQ23">
         <v>7.9080999999999995E-3</v>
       </c>
+      <c r="BR23">
+        <v>1.08047E-2</v>
+      </c>
+      <c r="BS23">
+        <v>7.9025999999999992E-3</v>
+      </c>
+      <c r="BT23">
+        <v>-1.0504100000000001E-2</v>
+      </c>
+      <c r="BU23">
+        <v>2.4603799999999999E-2</v>
+      </c>
+      <c r="BV23">
+        <v>1.4617E-2</v>
+      </c>
+      <c r="BW23">
+        <v>-3.9407400000000002E-2</v>
+      </c>
+      <c r="BX23">
+        <v>-4.5890800000000002E-2</v>
+      </c>
     </row>
-    <row r="24" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>274</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="C24" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D24">
         <v>-1.2888000000000001E-3</v>
@@ -6157,7 +6685,7 @@
         <v>0.17998259999999999</v>
       </c>
       <c r="Z24" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AA24">
         <v>7.1533600000000003E-2</v>
@@ -6288,13 +6816,34 @@
       <c r="BQ24">
         <v>2.7138900000000001E-2</v>
       </c>
+      <c r="BR24">
+        <v>3.6075E-3</v>
+      </c>
+      <c r="BS24">
+        <v>1.3506300000000001E-2</v>
+      </c>
+      <c r="BT24">
+        <v>7.5758000000000006E-2</v>
+      </c>
+      <c r="BU24">
+        <v>8.4124999999999998E-3</v>
+      </c>
+      <c r="BV24">
+        <v>3.7779899999999998E-2</v>
+      </c>
+      <c r="BW24">
+        <v>1.7347999999999999E-2</v>
+      </c>
+      <c r="BX24">
+        <v>1.5399100000000001E-2</v>
+      </c>
     </row>
-    <row r="25" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>1658</v>
       </c>
       <c r="C25" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D25">
         <v>-8.1019999999999996E-4</v>
@@ -6366,7 +6915,7 @@
         <v>-0.67374820000000002</v>
       </c>
       <c r="AA25" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AB25">
         <v>-0.58782279999999998</v>
@@ -6494,16 +7043,37 @@
       <c r="BQ25">
         <v>-2.9956E-2</v>
       </c>
+      <c r="BR25">
+        <v>2.0892999999999998E-2</v>
+      </c>
+      <c r="BS25">
+        <v>1.0786999999999999E-3</v>
+      </c>
+      <c r="BT25">
+        <v>-2.50073E-2</v>
+      </c>
+      <c r="BU25">
+        <v>2.4112700000000001E-2</v>
+      </c>
+      <c r="BV25">
+        <v>-9.0078999999999992E-3</v>
+      </c>
+      <c r="BW25">
+        <v>-8.8809399999999997E-2</v>
+      </c>
+      <c r="BX25">
+        <v>-5.6887699999999999E-2</v>
+      </c>
     </row>
-    <row r="26" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2072</v>
       </c>
       <c r="B26" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C26" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="D26">
         <v>1.9856000000000001E-3</v>
@@ -6578,7 +7148,7 @@
         <v>1.7479999999999999E-4</v>
       </c>
       <c r="AB26" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AC26">
         <v>-0.22975300000000001</v>
@@ -6703,16 +7273,37 @@
       <c r="BQ26">
         <v>1.45484E-2</v>
       </c>
+      <c r="BR26">
+        <v>1.13399E-2</v>
+      </c>
+      <c r="BS26">
+        <v>1.5548899999999999E-2</v>
+      </c>
+      <c r="BT26">
+        <v>3.06062E-2</v>
+      </c>
+      <c r="BU26">
+        <v>1.69616E-2</v>
+      </c>
+      <c r="BV26">
+        <v>-1.0646600000000001E-2</v>
+      </c>
+      <c r="BW26">
+        <v>3.0000999999999999E-3</v>
+      </c>
+      <c r="BX26">
+        <v>-1.2922999999999999E-3</v>
+      </c>
     </row>
-    <row r="27" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>1601</v>
       </c>
       <c r="B27" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C27" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D27">
         <v>-1.3035E-3</v>
@@ -6790,7 +7381,7 @@
         <v>-0.13916600000000001</v>
       </c>
       <c r="AC27" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AD27">
         <v>-0.1392207</v>
@@ -6912,16 +7503,37 @@
       <c r="BQ27">
         <v>2.7526200000000001E-2</v>
       </c>
+      <c r="BR27">
+        <v>3.48416E-2</v>
+      </c>
+      <c r="BS27">
+        <v>1.53052E-2</v>
+      </c>
+      <c r="BT27">
+        <v>2.2292300000000001E-2</v>
+      </c>
+      <c r="BU27">
+        <v>9.4109999999999992E-3</v>
+      </c>
+      <c r="BV27">
+        <v>1.17895E-2</v>
+      </c>
+      <c r="BW27">
+        <v>1.9482300000000001E-2</v>
+      </c>
+      <c r="BX27">
+        <v>1.0545000000000001E-3</v>
+      </c>
     </row>
-    <row r="28" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>445</v>
       </c>
       <c r="B28" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C28" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="D28">
         <v>-9.5960000000000001E-4</v>
@@ -7002,7 +7614,7 @@
         <v>-0.47284809999999999</v>
       </c>
       <c r="AD28" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AE28">
         <v>-0.4710432</v>
@@ -7121,16 +7733,37 @@
       <c r="BQ28">
         <v>2.3333999999999998E-3</v>
       </c>
+      <c r="BR28">
+        <v>3.5482399999999997E-2</v>
+      </c>
+      <c r="BS28">
+        <v>8.5892E-3</v>
+      </c>
+      <c r="BT28">
+        <v>-1.4868900000000001E-2</v>
+      </c>
+      <c r="BU28">
+        <v>9.7970000000000002E-3</v>
+      </c>
+      <c r="BV28">
+        <v>3.5048299999999998E-2</v>
+      </c>
+      <c r="BW28">
+        <v>2.42886E-2</v>
+      </c>
+      <c r="BX28">
+        <v>3.0462599999999999E-2</v>
+      </c>
     </row>
-    <row r="29" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>916</v>
       </c>
       <c r="B29" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="C29" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D29">
         <v>-2.1935000000000001E-3</v>
@@ -7214,7 +7847,7 @@
         <v>-0.34678829999999999</v>
       </c>
       <c r="AE29" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AF29">
         <v>1.2111E-2</v>
@@ -7330,13 +7963,34 @@
       <c r="BQ29">
         <v>1.2397200000000001E-2</v>
       </c>
+      <c r="BR29">
+        <v>5.2207E-3</v>
+      </c>
+      <c r="BS29">
+        <v>1.4762000000000001E-2</v>
+      </c>
+      <c r="BT29">
+        <v>-8.4005999999999994E-3</v>
+      </c>
+      <c r="BU29">
+        <v>1.07911E-2</v>
+      </c>
+      <c r="BV29">
+        <v>4.9822600000000002E-2</v>
+      </c>
+      <c r="BW29">
+        <v>-3.5766999999999999E-3</v>
+      </c>
+      <c r="BX29">
+        <v>9.8300000000000002E-3</v>
+      </c>
     </row>
-    <row r="30" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>53</v>
       </c>
       <c r="C30" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D30">
         <v>-6.5106000000000001E-3</v>
@@ -7423,7 +8077,7 @@
         <v>1.35502E-2</v>
       </c>
       <c r="AF30" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AG30">
         <v>-1.17316E-2</v>
@@ -7536,13 +8190,34 @@
       <c r="BQ30">
         <v>6.6722999999999999E-3</v>
       </c>
+      <c r="BR30">
+        <v>9.5007000000000008E-3</v>
+      </c>
+      <c r="BS30">
+        <v>1.20997E-2</v>
+      </c>
+      <c r="BT30">
+        <v>7.8310000000000001E-4</v>
+      </c>
+      <c r="BU30">
+        <v>1.3356E-2</v>
+      </c>
+      <c r="BV30">
+        <v>-6.9810000000000002E-3</v>
+      </c>
+      <c r="BW30">
+        <v>5.239E-4</v>
+      </c>
+      <c r="BX30">
+        <v>1.1408E-2</v>
+      </c>
     </row>
-    <row r="31" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>1526</v>
       </c>
       <c r="C31" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D31">
         <v>-6.3822000000000002E-3</v>
@@ -7632,7 +8307,7 @@
         <v>5.4997400000000002E-2</v>
       </c>
       <c r="AG31" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AH31">
         <v>1.2799400000000001E-2</v>
@@ -7742,13 +8417,34 @@
       <c r="BQ31">
         <v>3.4687200000000001E-2</v>
       </c>
+      <c r="BR31">
+        <v>1.493E-3</v>
+      </c>
+      <c r="BS31">
+        <v>1.0522699999999999E-2</v>
+      </c>
+      <c r="BT31">
+        <v>1.0755000000000001E-2</v>
+      </c>
+      <c r="BU31">
+        <v>1.7350999999999998E-2</v>
+      </c>
+      <c r="BV31">
+        <v>1.6117200000000002E-2</v>
+      </c>
+      <c r="BW31">
+        <v>2.2880399999999999E-2</v>
+      </c>
+      <c r="BX31">
+        <v>2.5145799999999999E-2</v>
+      </c>
     </row>
-    <row r="32" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>356</v>
       </c>
       <c r="C32" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D32">
         <v>-7.1494999999999996E-3</v>
@@ -7841,7 +8537,7 @@
         <v>3.7074700000000002E-2</v>
       </c>
       <c r="AH32" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AI32">
         <v>7.1173500000000001E-2</v>
@@ -7948,13 +8644,34 @@
       <c r="BQ32">
         <v>4.09425E-2</v>
       </c>
+      <c r="BR32">
+        <v>1.1682999999999999E-3</v>
+      </c>
+      <c r="BS32">
+        <v>9.7861000000000007E-3</v>
+      </c>
+      <c r="BT32">
+        <v>2.0478199999999998E-2</v>
+      </c>
+      <c r="BU32">
+        <v>1.69722E-2</v>
+      </c>
+      <c r="BV32">
+        <v>1.30803E-2</v>
+      </c>
+      <c r="BW32">
+        <v>1.9289500000000001E-2</v>
+      </c>
+      <c r="BX32">
+        <v>1.8294899999999999E-2</v>
+      </c>
     </row>
-    <row r="33" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>415</v>
       </c>
       <c r="C33" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D33">
         <v>-6.5547000000000001E-3</v>
@@ -8050,7 +8767,7 @@
         <v>1.3287200000000001E-2</v>
       </c>
       <c r="AI33" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AJ33">
         <v>2.2283899999999999E-2</v>
@@ -8154,13 +8871,34 @@
       <c r="BQ33">
         <v>2.3005600000000001E-2</v>
       </c>
+      <c r="BR33">
+        <v>1.7306000000000001E-3</v>
+      </c>
+      <c r="BS33">
+        <v>8.1455E-3</v>
+      </c>
+      <c r="BT33">
+        <v>1.3455E-2</v>
+      </c>
+      <c r="BU33">
+        <v>1.8461499999999999E-2</v>
+      </c>
+      <c r="BV33">
+        <v>7.4710000000000002E-3</v>
+      </c>
+      <c r="BW33">
+        <v>2.2714600000000001E-2</v>
+      </c>
+      <c r="BX33">
+        <v>1.59416E-2</v>
+      </c>
     </row>
-    <row r="34" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>1278</v>
       </c>
       <c r="C34" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D34">
         <v>-5.9473E-3</v>
@@ -8259,7 +8997,7 @@
         <v>7.8315300000000004E-2</v>
       </c>
       <c r="AJ34" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AK34">
         <v>0.1176919</v>
@@ -8360,13 +9098,34 @@
       <c r="BQ34">
         <v>3.1368500000000001E-2</v>
       </c>
+      <c r="BR34">
+        <v>4.8685600000000002E-2</v>
+      </c>
+      <c r="BS34">
+        <v>1.9379799999999999E-2</v>
+      </c>
+      <c r="BT34">
+        <v>2.00544E-2</v>
+      </c>
+      <c r="BU34">
+        <v>2.4166099999999999E-2</v>
+      </c>
+      <c r="BV34">
+        <v>5.2324700000000002E-2</v>
+      </c>
+      <c r="BW34">
+        <v>8.1531099999999995E-2</v>
+      </c>
+      <c r="BX34">
+        <v>6.1573700000000002E-2</v>
+      </c>
     </row>
-    <row r="35" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>2394</v>
       </c>
       <c r="C35" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D35">
         <v>-6.4031000000000001E-3</v>
@@ -8468,7 +9227,7 @@
         <v>6.4736600000000005E-2</v>
       </c>
       <c r="AK35" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AL35">
         <v>4.3137399999999999E-2</v>
@@ -8566,13 +9325,34 @@
       <c r="BQ35">
         <v>2.6493699999999999E-2</v>
       </c>
+      <c r="BR35">
+        <v>4.4948999999999996E-3</v>
+      </c>
+      <c r="BS35">
+        <v>1.0090200000000001E-2</v>
+      </c>
+      <c r="BT35">
+        <v>1.77498E-2</v>
+      </c>
+      <c r="BU35">
+        <v>1.4977900000000001E-2</v>
+      </c>
+      <c r="BV35">
+        <v>1.3845100000000001E-2</v>
+      </c>
+      <c r="BW35">
+        <v>1.05237E-2</v>
+      </c>
+      <c r="BX35">
+        <v>3.32222E-2</v>
+      </c>
     </row>
-    <row r="36" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>1750</v>
       </c>
       <c r="C36" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D36">
         <v>-6.6433999999999998E-3</v>
@@ -8677,7 +9457,7 @@
         <v>6.3616300000000001E-2</v>
       </c>
       <c r="AL36" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AM36">
         <v>7.5059500000000001E-2</v>
@@ -8772,13 +9552,34 @@
       <c r="BQ36">
         <v>3.1919999999999997E-2</v>
       </c>
+      <c r="BR36">
+        <v>1.0023E-3</v>
+      </c>
+      <c r="BS36">
+        <v>9.3650999999999995E-3</v>
+      </c>
+      <c r="BT36">
+        <v>1.38254E-2</v>
+      </c>
+      <c r="BU36">
+        <v>1.34036E-2</v>
+      </c>
+      <c r="BV36">
+        <v>1.9433E-3</v>
+      </c>
+      <c r="BW36">
+        <v>6.4993000000000004E-3</v>
+      </c>
+      <c r="BX36">
+        <v>9.2791000000000002E-3</v>
+      </c>
     </row>
-    <row r="37" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>150</v>
       </c>
       <c r="C37" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D37">
         <v>-6.4659000000000001E-3</v>
@@ -8886,7 +9687,7 @@
         <v>3.9029500000000002E-2</v>
       </c>
       <c r="AM37" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AN37">
         <v>1.19208E-2</v>
@@ -8978,13 +9779,34 @@
       <c r="BQ37">
         <v>3.39548E-2</v>
       </c>
+      <c r="BR37">
+        <v>2.9100000000000003E-4</v>
+      </c>
+      <c r="BS37">
+        <v>1.23803E-2</v>
+      </c>
+      <c r="BT37">
+        <v>7.9167000000000005E-3</v>
+      </c>
+      <c r="BU37">
+        <v>1.59731E-2</v>
+      </c>
+      <c r="BV37">
+        <v>-1.1498999999999999E-3</v>
+      </c>
+      <c r="BW37">
+        <v>1.00156E-2</v>
+      </c>
+      <c r="BX37">
+        <v>1.1946999999999999E-2</v>
+      </c>
     </row>
-    <row r="38" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>728</v>
       </c>
       <c r="C38" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="D38">
         <v>-5.8566E-3</v>
@@ -9095,7 +9917,7 @@
         <v>-0.1067676</v>
       </c>
       <c r="AN38" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AO38">
         <v>-0.55194960000000004</v>
@@ -9184,13 +10006,34 @@
       <c r="BQ38">
         <v>-1.6761999999999999E-2</v>
       </c>
+      <c r="BR38">
+        <v>-1.2926699999999999E-2</v>
+      </c>
+      <c r="BS38">
+        <v>-8.2179999999999996E-3</v>
+      </c>
+      <c r="BT38">
+        <v>-2.1884799999999999E-2</v>
+      </c>
+      <c r="BU38">
+        <v>1.0591400000000001E-2</v>
+      </c>
+      <c r="BV38">
+        <v>-6.0879900000000001E-2</v>
+      </c>
+      <c r="BW38">
+        <v>-7.4999899999999994E-2</v>
+      </c>
+      <c r="BX38">
+        <v>-3.2647700000000002E-2</v>
+      </c>
     </row>
-    <row r="39" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>312</v>
       </c>
       <c r="C39" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D39">
         <v>-5.4057999999999997E-3</v>
@@ -9304,7 +10147,7 @@
         <v>-1.32248E-2</v>
       </c>
       <c r="AO39" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AP39">
         <v>-1.0196999999999999E-2</v>
@@ -9390,13 +10233,34 @@
       <c r="BQ39">
         <v>2.7085999999999999E-2</v>
       </c>
+      <c r="BR39">
+        <v>8.1071000000000008E-3</v>
+      </c>
+      <c r="BS39">
+        <v>-3.6143999999999998E-3</v>
+      </c>
+      <c r="BT39">
+        <v>9.3407999999999998E-3</v>
+      </c>
+      <c r="BU39">
+        <v>1.6605600000000002E-2</v>
+      </c>
+      <c r="BV39">
+        <v>-1.7601100000000001E-2</v>
+      </c>
+      <c r="BW39">
+        <v>-2.2571299999999999E-2</v>
+      </c>
+      <c r="BX39">
+        <v>-1.8218100000000001E-2</v>
+      </c>
     </row>
-    <row r="40" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D40">
         <v>-6.6537999999999996E-3</v>
@@ -9513,7 +10377,7 @@
         <v>3.0092299999999999E-2</v>
       </c>
       <c r="AP40" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AQ40">
         <v>3.2548100000000003E-2</v>
@@ -9596,13 +10460,34 @@
       <c r="BQ40">
         <v>1.24391E-2</v>
       </c>
+      <c r="BR40">
+        <v>3.8365000000000001E-3</v>
+      </c>
+      <c r="BS40">
+        <v>9.4307999999999996E-3</v>
+      </c>
+      <c r="BT40">
+        <v>8.8123999999999997E-3</v>
+      </c>
+      <c r="BU40">
+        <v>5.5957000000000003E-3</v>
+      </c>
+      <c r="BV40">
+        <v>2.1310000000000001E-3</v>
+      </c>
+      <c r="BW40">
+        <v>-2.4291699999999999E-2</v>
+      </c>
+      <c r="BX40">
+        <v>-5.9715000000000002E-3</v>
+      </c>
     </row>
-    <row r="41" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A41">
         <v>392</v>
       </c>
       <c r="C41" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="D41">
         <v>-6.7774000000000003E-3</v>
@@ -9722,7 +10607,7 @@
         <v>1.33107E-2</v>
       </c>
       <c r="AQ41" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AR41">
         <v>5.5249100000000002E-2</v>
@@ -9802,13 +10687,34 @@
       <c r="BQ41">
         <v>3.2321000000000003E-2</v>
       </c>
+      <c r="BR41">
+        <v>-2.7858000000000002E-3</v>
+      </c>
+      <c r="BS41">
+        <v>9.2204000000000001E-3</v>
+      </c>
+      <c r="BT41">
+        <v>1.0187099999999999E-2</v>
+      </c>
+      <c r="BU41">
+        <v>1.93026E-2</v>
+      </c>
+      <c r="BV41">
+        <v>1.8169E-3</v>
+      </c>
+      <c r="BW41">
+        <v>7.8904000000000005E-3</v>
+      </c>
+      <c r="BX41">
+        <v>1.04466E-2</v>
+      </c>
     </row>
-    <row r="42" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>1346</v>
       </c>
       <c r="C42" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D42">
         <v>-6.149E-3</v>
@@ -9931,7 +10837,7 @@
         <v>1.0474300000000001E-2</v>
       </c>
       <c r="AR42" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AS42">
         <v>2.96213E-2</v>
@@ -10008,16 +10914,37 @@
       <c r="BQ42" s="1">
         <v>9.6399999999999999E-5</v>
       </c>
+      <c r="BR42">
+        <v>4.8353100000000003E-2</v>
+      </c>
+      <c r="BS42">
+        <v>1.3745500000000001E-2</v>
+      </c>
+      <c r="BT42">
+        <v>-2.5818399999999998E-2</v>
+      </c>
+      <c r="BU42">
+        <v>1.48643E-2</v>
+      </c>
+      <c r="BV42">
+        <v>1.6312900000000002E-2</v>
+      </c>
+      <c r="BW42">
+        <v>2.4266200000000002E-2</v>
+      </c>
+      <c r="BX42">
+        <v>4.3122500000000001E-2</v>
+      </c>
     </row>
-    <row r="43" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1466</v>
       </c>
       <c r="B43" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C43" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D43">
         <v>-8.1279000000000004E-3</v>
@@ -10143,7 +11070,7 @@
         <v>5.4456299999999999E-2</v>
       </c>
       <c r="AS43" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AT43">
         <v>-0.17780699999999999</v>
@@ -10217,16 +11144,37 @@
       <c r="BQ43">
         <v>2.2619299999999998E-2</v>
       </c>
+      <c r="BR43">
+        <v>-1.9443999999999999E-2</v>
+      </c>
+      <c r="BS43">
+        <v>1.0173400000000001E-2</v>
+      </c>
+      <c r="BT43">
+        <v>8.0514999999999996E-3</v>
+      </c>
+      <c r="BU43">
+        <v>1.7012900000000001E-2</v>
+      </c>
+      <c r="BV43">
+        <v>1.6791500000000001E-2</v>
+      </c>
+      <c r="BW43">
+        <v>4.3578600000000002E-2</v>
+      </c>
+      <c r="BX43">
+        <v>1.8482200000000001E-2</v>
+      </c>
     </row>
-    <row r="44" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1588</v>
       </c>
       <c r="B44" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C44" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="D44">
         <v>-7.2951999999999999E-3</v>
@@ -10355,7 +11303,7 @@
         <v>-0.26802369999999998</v>
       </c>
       <c r="AT44" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AU44">
         <v>-0.1796509</v>
@@ -10426,16 +11374,37 @@
       <c r="BQ44">
         <v>2.6307400000000002E-2</v>
       </c>
+      <c r="BR44">
+        <v>-2.6547999999999999E-2</v>
+      </c>
+      <c r="BS44">
+        <v>9.2642000000000002E-3</v>
+      </c>
+      <c r="BT44">
+        <v>3.5775E-3</v>
+      </c>
+      <c r="BU44">
+        <v>1.4167300000000001E-2</v>
+      </c>
+      <c r="BV44">
+        <v>9.3898999999999996E-3</v>
+      </c>
+      <c r="BW44">
+        <v>5.95831E-2</v>
+      </c>
+      <c r="BX44">
+        <v>-8.5836000000000003E-3</v>
+      </c>
     </row>
-    <row r="45" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>1048</v>
       </c>
       <c r="B45" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C45" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D45">
         <v>-4.3616999999999996E-3</v>
@@ -10567,7 +11536,7 @@
         <v>-0.36866850000000001</v>
       </c>
       <c r="AU45" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AV45">
         <v>-0.28122049999999998</v>
@@ -10635,16 +11604,37 @@
       <c r="BQ45">
         <v>-8.1033000000000008E-3</v>
       </c>
+      <c r="BR45">
+        <v>-6.0007999999999997E-3</v>
+      </c>
+      <c r="BS45">
+        <v>1.0203200000000001E-2</v>
+      </c>
+      <c r="BT45">
+        <v>-7.2874000000000003E-3</v>
+      </c>
+      <c r="BU45">
+        <v>1.36781E-2</v>
+      </c>
+      <c r="BV45">
+        <v>1.9766700000000002E-2</v>
+      </c>
+      <c r="BW45">
+        <v>4.22405E-2</v>
+      </c>
+      <c r="BX45">
+        <v>-3.4824999999999999E-3</v>
+      </c>
     </row>
-    <row r="46" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>2029</v>
       </c>
       <c r="B46" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C46" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D46">
         <v>-5.5300999999999996E-3</v>
@@ -10779,7 +11769,7 @@
         <v>-3.66205E-2</v>
       </c>
       <c r="AV46" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AW46">
         <v>-6.0102299999999997E-2</v>
@@ -10844,16 +11834,37 @@
       <c r="BQ46">
         <v>1.9280700000000001E-2</v>
       </c>
+      <c r="BR46">
+        <v>-2.0672800000000002E-2</v>
+      </c>
+      <c r="BS46">
+        <v>3.6235E-3</v>
+      </c>
+      <c r="BT46">
+        <v>-1.6151100000000002E-2</v>
+      </c>
+      <c r="BU46">
+        <v>-7.8129999999999996E-4</v>
+      </c>
+      <c r="BV46">
+        <v>-6.1743899999999997E-2</v>
+      </c>
+      <c r="BW46">
+        <v>-7.9319999999999998E-4</v>
+      </c>
+      <c r="BX46">
+        <v>2.0569799999999999E-2</v>
+      </c>
     </row>
-    <row r="47" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>1860</v>
       </c>
       <c r="B47" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C47" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D47">
         <v>-8.7481999999999994E-3</v>
@@ -10991,7 +12002,7 @@
         <v>-0.10584109999999999</v>
       </c>
       <c r="AW47" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AX47">
         <v>-0.1183152</v>
@@ -11053,16 +12064,37 @@
       <c r="BQ47">
         <v>2.35467E-2</v>
       </c>
+      <c r="BR47">
+        <v>-2.2131399999999999E-2</v>
+      </c>
+      <c r="BS47">
+        <v>1.3742000000000001E-2</v>
+      </c>
+      <c r="BT47">
+        <v>7.9647999999999993E-3</v>
+      </c>
+      <c r="BU47">
+        <v>2.2099899999999999E-2</v>
+      </c>
+      <c r="BV47">
+        <v>1.5482599999999999E-2</v>
+      </c>
+      <c r="BW47">
+        <v>4.6729800000000002E-2</v>
+      </c>
+      <c r="BX47">
+        <v>7.8178999999999992E-3</v>
+      </c>
     </row>
-    <row r="48" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>601</v>
       </c>
       <c r="B48" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="C48" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D48">
         <v>-7.2528000000000002E-3</v>
@@ -11203,7 +12235,7 @@
         <v>-0.30453380000000002</v>
       </c>
       <c r="AX48" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AY48">
         <v>-0.22051229999999999</v>
@@ -11262,13 +12294,34 @@
       <c r="BQ48">
         <v>-8.3730000000000002E-3</v>
       </c>
+      <c r="BR48">
+        <v>-7.8201E-3</v>
+      </c>
+      <c r="BS48">
+        <v>7.8203999999999999E-3</v>
+      </c>
+      <c r="BT48">
+        <v>-1.7252799999999999E-2</v>
+      </c>
+      <c r="BU48">
+        <v>9.6273999999999995E-3</v>
+      </c>
+      <c r="BV48">
+        <v>8.3782000000000006E-3</v>
+      </c>
+      <c r="BW48">
+        <v>-3.9071099999999997E-2</v>
+      </c>
+      <c r="BX48">
+        <v>-2.3154999999999999E-2</v>
+      </c>
     </row>
-    <row r="49" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>564</v>
       </c>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D49">
         <v>-7.3961000000000001E-3</v>
@@ -11412,7 +12465,7 @@
         <v>-0.1794829</v>
       </c>
       <c r="AY49" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="AZ49">
         <v>7.2870000000000001E-3</v>
@@ -11468,13 +12521,34 @@
       <c r="BQ49">
         <v>1.11308E-2</v>
       </c>
+      <c r="BR49">
+        <v>-2.9322500000000001E-2</v>
+      </c>
+      <c r="BS49">
+        <v>7.2309999999999996E-3</v>
+      </c>
+      <c r="BT49">
+        <v>-9.0335999999999993E-3</v>
+      </c>
+      <c r="BU49">
+        <v>1.19174E-2</v>
+      </c>
+      <c r="BV49">
+        <v>-1.38447E-2</v>
+      </c>
+      <c r="BW49">
+        <v>3.7956200000000002E-2</v>
+      </c>
+      <c r="BX49">
+        <v>-1.58452E-2</v>
+      </c>
     </row>
-    <row r="50" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>1290</v>
       </c>
       <c r="C50" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D50">
         <v>-6.5408000000000003E-3</v>
@@ -11621,7 +12695,7 @@
         <v>6.7184099999999997E-2</v>
       </c>
       <c r="AZ50" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BA50">
         <v>2.7330299999999998E-2</v>
@@ -11674,13 +12748,34 @@
       <c r="BQ50">
         <v>3.3056299999999997E-2</v>
       </c>
+      <c r="BR50">
+        <v>-4.751E-3</v>
+      </c>
+      <c r="BS50">
+        <v>8.6303000000000005E-3</v>
+      </c>
+      <c r="BT50">
+        <v>7.9778999999999996E-3</v>
+      </c>
+      <c r="BU50">
+        <v>1.3781399999999999E-2</v>
+      </c>
+      <c r="BV50">
+        <v>5.4492999999999998E-3</v>
+      </c>
+      <c r="BW50">
+        <v>1.0175999999999999E-2</v>
+      </c>
+      <c r="BX50">
+        <v>1.18452E-2</v>
+      </c>
     </row>
-    <row r="51" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>4077</v>
       </c>
       <c r="C51" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D51">
         <v>-1.03112E-2</v>
@@ -11830,7 +12925,7 @@
         <v>5.8141400000000003E-2</v>
       </c>
       <c r="BA51" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BB51">
         <v>1.25367E-2</v>
@@ -11880,13 +12975,34 @@
       <c r="BQ51">
         <v>3.5748799999999997E-2</v>
       </c>
+      <c r="BR51">
+        <v>5.8951000000000003E-3</v>
+      </c>
+      <c r="BS51">
+        <v>9.0495000000000003E-3</v>
+      </c>
+      <c r="BT51">
+        <v>4.2129300000000001E-2</v>
+      </c>
+      <c r="BU51">
+        <v>1.7744599999999999E-2</v>
+      </c>
+      <c r="BV51">
+        <v>2.33464E-2</v>
+      </c>
+      <c r="BW51">
+        <v>1.9264400000000001E-2</v>
+      </c>
+      <c r="BX51">
+        <v>2.6386099999999999E-2</v>
+      </c>
     </row>
-    <row r="52" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>2436</v>
       </c>
       <c r="C52" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D52">
         <v>-7.5255000000000001E-3</v>
@@ -12039,7 +13155,7 @@
         <v>1.36683E-2</v>
       </c>
       <c r="BB52" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BC52">
         <v>4.9235599999999997E-2</v>
@@ -12086,16 +13202,37 @@
       <c r="BQ52">
         <v>3.3761100000000002E-2</v>
       </c>
+      <c r="BR52">
+        <v>-8.0771999999999997E-3</v>
+      </c>
+      <c r="BS52">
+        <v>1.06344E-2</v>
+      </c>
+      <c r="BT52">
+        <v>1.9358899999999998E-2</v>
+      </c>
+      <c r="BU52">
+        <v>1.9611900000000002E-2</v>
+      </c>
+      <c r="BV52">
+        <v>2.0582199999999998E-2</v>
+      </c>
+      <c r="BW52">
+        <v>3.6686200000000002E-2</v>
+      </c>
+      <c r="BX52">
+        <v>1.6531299999999999E-2</v>
+      </c>
     </row>
-    <row r="53" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>2106</v>
       </c>
       <c r="B53" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D53">
         <v>-6.5355999999999999E-3</v>
@@ -12251,7 +13388,7 @@
         <v>1.5622499999999999E-2</v>
       </c>
       <c r="BC53" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BD53">
         <v>5.4039999999999999E-3</v>
@@ -12295,16 +13432,37 @@
       <c r="BQ53">
         <v>3.4803000000000001E-2</v>
       </c>
+      <c r="BR53">
+        <v>-5.2328000000000001E-3</v>
+      </c>
+      <c r="BS53">
+        <v>0.01</v>
+      </c>
+      <c r="BT53">
+        <v>9.5364999999999998E-3</v>
+      </c>
+      <c r="BU53">
+        <v>1.8778199999999998E-2</v>
+      </c>
+      <c r="BV53">
+        <v>6.2430000000000003E-3</v>
+      </c>
+      <c r="BW53">
+        <v>5.3439000000000004E-3</v>
+      </c>
+      <c r="BX53">
+        <v>1.5334199999999999E-2</v>
+      </c>
     </row>
-    <row r="54" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>1512</v>
       </c>
       <c r="B54" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C54" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="D54">
         <v>-7.4484E-3</v>
@@ -12463,7 +13621,7 @@
         <v>3.5126900000000003E-2</v>
       </c>
       <c r="BD54" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BE54">
         <v>-1.0861300000000001E-2</v>
@@ -12504,16 +13662,37 @@
       <c r="BQ54">
         <v>3.3547800000000003E-2</v>
       </c>
+      <c r="BR54">
+        <v>-6.2316000000000003E-3</v>
+      </c>
+      <c r="BS54">
+        <v>9.3962999999999998E-3</v>
+      </c>
+      <c r="BT54">
+        <v>2.7687799999999999E-2</v>
+      </c>
+      <c r="BU54">
+        <v>1.95684E-2</v>
+      </c>
+      <c r="BV54">
+        <v>1.77614E-2</v>
+      </c>
+      <c r="BW54">
+        <v>2.38458E-2</v>
+      </c>
+      <c r="BX54">
+        <v>1.3202E-2</v>
+      </c>
     </row>
-    <row r="55" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>2456</v>
       </c>
       <c r="B55" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C55" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D55">
         <v>-7.6544999999999998E-3</v>
@@ -12675,7 +13854,7 @@
         <v>-9.4798E-3</v>
       </c>
       <c r="BE55" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BF55">
         <v>1.35367E-2</v>
@@ -12713,16 +13892,37 @@
       <c r="BQ55">
         <v>3.6495199999999998E-2</v>
       </c>
+      <c r="BR55">
+        <v>-8.7627999999999994E-3</v>
+      </c>
+      <c r="BS55">
+        <v>1.23074E-2</v>
+      </c>
+      <c r="BT55">
+        <v>2.5305399999999999E-2</v>
+      </c>
+      <c r="BU55">
+        <v>1.7873699999999999E-2</v>
+      </c>
+      <c r="BV55">
+        <v>1.13191E-2</v>
+      </c>
+      <c r="BW55">
+        <v>2.67663E-2</v>
+      </c>
+      <c r="BX55">
+        <v>1.7412299999999999E-2</v>
+      </c>
     </row>
-    <row r="56" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>1204</v>
       </c>
       <c r="B56" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C56" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D56">
         <v>-7.2794000000000001E-3</v>
@@ -12887,7 +14087,7 @@
         <v>-1.1781000000000001E-3</v>
       </c>
       <c r="BF56" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BG56">
         <v>1.4604600000000001E-2</v>
@@ -12922,16 +14122,37 @@
       <c r="BQ56">
         <v>3.6986699999999997E-2</v>
       </c>
+      <c r="BR56">
+        <v>-3.8514999999999999E-3</v>
+      </c>
+      <c r="BS56">
+        <v>9.5286999999999993E-3</v>
+      </c>
+      <c r="BT56">
+        <v>1.65959E-2</v>
+      </c>
+      <c r="BU56">
+        <v>1.8536299999999999E-2</v>
+      </c>
+      <c r="BV56">
+        <v>7.5538999999999997E-3</v>
+      </c>
+      <c r="BW56">
+        <v>1.0981299999999999E-2</v>
+      </c>
+      <c r="BX56">
+        <v>1.40888E-2</v>
+      </c>
     </row>
-    <row r="57" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>952</v>
       </c>
       <c r="B57" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="C57" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="D57">
         <v>-7.1406000000000004E-3</v>
@@ -13099,7 +14320,7 @@
         <v>1.3639399999999999E-2</v>
       </c>
       <c r="BG57" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BH57">
         <v>1.2578600000000001E-2</v>
@@ -13131,16 +14352,37 @@
       <c r="BQ57">
         <v>3.3258900000000001E-2</v>
       </c>
+      <c r="BR57">
+        <v>-3.6717E-3</v>
+      </c>
+      <c r="BS57">
+        <v>8.7588000000000006E-3</v>
+      </c>
+      <c r="BT57">
+        <v>1.2393299999999999E-2</v>
+      </c>
+      <c r="BU57">
+        <v>1.5470899999999999E-2</v>
+      </c>
+      <c r="BV57">
+        <v>5.6944999999999999E-3</v>
+      </c>
+      <c r="BW57">
+        <v>1.2588500000000001E-2</v>
+      </c>
+      <c r="BX57">
+        <v>1.09839E-2</v>
+      </c>
     </row>
-    <row r="58" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A58">
         <v>2245</v>
       </c>
       <c r="B58" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C58" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D58">
         <v>-5.2893000000000003E-3</v>
@@ -13311,7 +14553,7 @@
         <v>-5.3053099999999999E-2</v>
       </c>
       <c r="BH58" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BI58">
         <v>-0.147091</v>
@@ -13340,16 +14582,37 @@
       <c r="BQ58">
         <v>4.3952499999999999E-2</v>
       </c>
+      <c r="BR58">
+        <v>-1.0869200000000001E-2</v>
+      </c>
+      <c r="BS58">
+        <v>9.6358999999999993E-3</v>
+      </c>
+      <c r="BT58">
+        <v>3.5298000000000003E-2</v>
+      </c>
+      <c r="BU58">
+        <v>2.1523199999999999E-2</v>
+      </c>
+      <c r="BV58">
+        <v>-2.13501E-2</v>
+      </c>
+      <c r="BW58">
+        <v>5.7920999999999997E-3</v>
+      </c>
+      <c r="BX58">
+        <v>1.0926699999999999E-2</v>
+      </c>
     </row>
-    <row r="59" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A59">
         <v>793</v>
       </c>
       <c r="B59" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="C59" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="D59">
         <v>-8.5134000000000008E-3</v>
@@ -13523,7 +14786,7 @@
         <v>1.0600999999999999E-2</v>
       </c>
       <c r="BI59" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BJ59">
         <v>-4.2703400000000002E-2</v>
@@ -13549,13 +14812,34 @@
       <c r="BQ59">
         <v>4.5106599999999997E-2</v>
       </c>
+      <c r="BR59">
+        <v>-2.2134399999999999E-2</v>
+      </c>
+      <c r="BS59">
+        <v>9.2461000000000002E-3</v>
+      </c>
+      <c r="BT59">
+        <v>2.88063E-2</v>
+      </c>
+      <c r="BU59">
+        <v>2.2685799999999999E-2</v>
+      </c>
+      <c r="BV59">
+        <v>-6.9251E-3</v>
+      </c>
+      <c r="BW59">
+        <v>2.5884600000000001E-2</v>
+      </c>
+      <c r="BX59">
+        <v>2.8576799999999999E-2</v>
+      </c>
     </row>
-    <row r="60" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A60">
         <v>3180</v>
       </c>
       <c r="C60" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="D60">
         <v>3.7921999999999999E-3</v>
@@ -13732,7 +15016,7 @@
         <v>-8.1990400000000005E-2</v>
       </c>
       <c r="BJ60" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BK60">
         <v>-0.1025947</v>
@@ -13755,13 +15039,34 @@
       <c r="BQ60">
         <v>5.8154900000000002E-2</v>
       </c>
+      <c r="BR60">
+        <v>4.2022200000000003E-2</v>
+      </c>
+      <c r="BS60">
+        <v>2.5366E-3</v>
+      </c>
+      <c r="BT60">
+        <v>-0.12388209999999999</v>
+      </c>
+      <c r="BU60">
+        <v>2.7199999999999998E-2</v>
+      </c>
+      <c r="BV60">
+        <v>-0.16649330000000001</v>
+      </c>
+      <c r="BW60">
+        <v>2.21628E-2</v>
+      </c>
+      <c r="BX60">
+        <v>-0.10344150000000001</v>
+      </c>
     </row>
-    <row r="61" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A61">
         <v>612</v>
       </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D61">
         <v>-2.1542000000000002E-3</v>
@@ -13941,7 +15246,7 @@
         <v>-3.1401699999999998E-2</v>
       </c>
       <c r="BK61" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BL61">
         <v>-0.20589969999999999</v>
@@ -13961,16 +15266,37 @@
       <c r="BQ61">
         <v>-6.9086E-3</v>
       </c>
+      <c r="BR61">
+        <v>-0.13627449999999999</v>
+      </c>
+      <c r="BS61">
+        <v>4.22499E-2</v>
+      </c>
+      <c r="BT61">
+        <v>-6.4106399999999994E-2</v>
+      </c>
+      <c r="BU61">
+        <v>5.0502600000000002E-2</v>
+      </c>
+      <c r="BV61">
+        <v>-9.8820400000000003E-2</v>
+      </c>
+      <c r="BW61">
+        <v>1.5715E-3</v>
+      </c>
+      <c r="BX61">
+        <v>-2.5885600000000002E-2</v>
+      </c>
     </row>
-    <row r="62" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A62">
         <v>2451</v>
       </c>
       <c r="B62" t="s">
+        <v>157</v>
+      </c>
+      <c r="C62" t="s">
         <v>136</v>
-      </c>
-      <c r="C62" t="s">
-        <v>129</v>
       </c>
       <c r="D62">
         <v>5.9845999999999996E-3</v>
@@ -14153,7 +15479,7 @@
         <v>-0.33472550000000001</v>
       </c>
       <c r="BL62" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BM62">
         <v>-0.28152700000000003</v>
@@ -14170,16 +15496,37 @@
       <c r="BQ62">
         <v>-4.2542999999999997E-2</v>
       </c>
+      <c r="BR62">
+        <v>-0.14108660000000001</v>
+      </c>
+      <c r="BS62">
+        <v>2.4565099999999999E-2</v>
+      </c>
+      <c r="BT62">
+        <v>-0.1633117</v>
+      </c>
+      <c r="BU62">
+        <v>1.17251E-2</v>
+      </c>
+      <c r="BV62">
+        <v>-0.17661450000000001</v>
+      </c>
+      <c r="BW62">
+        <v>-5.6047100000000002E-2</v>
+      </c>
+      <c r="BX62">
+        <v>-5.8929299999999997E-2</v>
+      </c>
     </row>
-    <row r="63" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>215</v>
       </c>
       <c r="B63" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C63" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="D63">
         <v>1.593E-3</v>
@@ -14365,7 +15712,7 @@
         <v>0.1100064</v>
       </c>
       <c r="BM63" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BN63">
         <v>8.5670899999999994E-2</v>
@@ -14379,16 +15726,37 @@
       <c r="BQ63">
         <v>1.9720100000000001E-2</v>
       </c>
+      <c r="BR63">
+        <v>-7.4597999999999999E-3</v>
+      </c>
+      <c r="BS63">
+        <v>0.10303420000000001</v>
+      </c>
+      <c r="BT63">
+        <v>-2.4444500000000001E-2</v>
+      </c>
+      <c r="BU63">
+        <v>7.0064699999999994E-2</v>
+      </c>
+      <c r="BV63">
+        <v>2.5806599999999999E-2</v>
+      </c>
+      <c r="BW63">
+        <v>0.1047332</v>
+      </c>
+      <c r="BX63">
+        <v>6.9141900000000006E-2</v>
+      </c>
     </row>
-    <row r="64" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>1683</v>
       </c>
       <c r="B64" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C64" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D64">
         <v>1.9566000000000002E-3</v>
@@ -14577,7 +15945,7 @@
         <v>-0.2585442</v>
       </c>
       <c r="BN64" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BO64">
         <v>-0.37937460000000001</v>
@@ -14588,16 +15956,37 @@
       <c r="BQ64">
         <v>-1.84222E-2</v>
       </c>
+      <c r="BR64">
+        <v>-0.1526371</v>
+      </c>
+      <c r="BS64">
+        <v>4.3304000000000002E-2</v>
+      </c>
+      <c r="BT64">
+        <v>-8.5128899999999993E-2</v>
+      </c>
+      <c r="BU64">
+        <v>2.2690399999999999E-2</v>
+      </c>
+      <c r="BV64">
+        <v>-0.12633829999999999</v>
+      </c>
+      <c r="BW64">
+        <v>-3.7092399999999998E-2</v>
+      </c>
+      <c r="BX64">
+        <v>-3.5290200000000001E-2</v>
+      </c>
     </row>
-    <row r="65" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>1948</v>
       </c>
       <c r="B65" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="C65" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="D65">
         <v>3.8704E-3</v>
@@ -14789,7 +16178,7 @@
         <v>1.2019E-2</v>
       </c>
       <c r="BO65" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BP65">
         <v>3.1527E-3</v>
@@ -14797,16 +16186,37 @@
       <c r="BQ65">
         <v>1.3111899999999999E-2</v>
       </c>
+      <c r="BR65">
+        <v>-0.10014380000000001</v>
+      </c>
+      <c r="BS65">
+        <v>6.1097800000000001E-2</v>
+      </c>
+      <c r="BT65">
+        <v>-5.1676899999999998E-2</v>
+      </c>
+      <c r="BU65">
+        <v>3.7654800000000002E-2</v>
+      </c>
+      <c r="BV65">
+        <v>-2.2462300000000001E-2</v>
+      </c>
+      <c r="BW65">
+        <v>2.7279899999999999E-2</v>
+      </c>
+      <c r="BX65">
+        <v>3.8169000000000002E-2</v>
+      </c>
     </row>
-    <row r="66" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>203</v>
       </c>
       <c r="B66" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C66" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D66">
         <v>-6.816E-3</v>
@@ -15001,21 +16411,42 @@
         <v>-3.9966999999999997E-3</v>
       </c>
       <c r="BP66" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="BQ66">
         <v>1.8310300000000002E-2</v>
       </c>
+      <c r="BR66">
+        <v>-6.9854000000000001E-3</v>
+      </c>
+      <c r="BS66">
+        <v>1.94842E-2</v>
+      </c>
+      <c r="BT66">
+        <v>2.8503000000000001E-3</v>
+      </c>
+      <c r="BU66">
+        <v>3.1896399999999998E-2</v>
+      </c>
+      <c r="BV66">
+        <v>8.6303000000000005E-3</v>
+      </c>
+      <c r="BW66">
+        <v>6.8699E-3</v>
+      </c>
+      <c r="BX66">
+        <v>2.6708599999999999E-2</v>
+      </c>
     </row>
-    <row r="67" spans="1:69" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:76" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>1047</v>
       </c>
       <c r="B67" t="s">
-        <v>137</v>
+        <v>158</v>
       </c>
       <c r="C67" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="D67">
         <v>-7.9027999999999998E-3</v>
@@ -15213,23 +16644,1648 @@
         <v>1.5306699999999999E-2</v>
       </c>
       <c r="BQ67" t="s">
-        <v>69</v>
+        <v>76</v>
+      </c>
+      <c r="BR67">
+        <v>1.6685999999999999E-3</v>
+      </c>
+      <c r="BS67">
+        <v>-3.7948999999999999E-3</v>
+      </c>
+      <c r="BT67">
+        <v>5.7771000000000003E-3</v>
+      </c>
+      <c r="BU67">
+        <v>2.7944E-2</v>
+      </c>
+      <c r="BV67">
+        <v>5.7784999999999998E-3</v>
+      </c>
+      <c r="BW67">
+        <v>5.8436099999999998E-2</v>
+      </c>
+      <c r="BX67">
+        <v>5.8142800000000001E-2</v>
+      </c>
+    </row>
+    <row r="68" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>1570</v>
+      </c>
+      <c r="C68" t="s">
+        <v>142</v>
+      </c>
+      <c r="D68">
+        <v>8.2302E-3</v>
+      </c>
+      <c r="E68">
+        <v>6.4136000000000002E-3</v>
+      </c>
+      <c r="F68" s="1">
+        <v>8.03E-5</v>
+      </c>
+      <c r="G68">
+        <v>2.7705199999999999E-2</v>
+      </c>
+      <c r="H68">
+        <v>3.8530999999999999E-3</v>
+      </c>
+      <c r="I68">
+        <v>5.4267999999999999E-3</v>
+      </c>
+      <c r="J68">
+        <v>6.6445000000000002E-3</v>
+      </c>
+      <c r="K68">
+        <v>4.2621699999999998E-2</v>
+      </c>
+      <c r="L68">
+        <v>4.8770599999999997E-2</v>
+      </c>
+      <c r="M68">
+        <v>0.1696608</v>
+      </c>
+      <c r="N68">
+        <v>0.16586229999999999</v>
+      </c>
+      <c r="O68">
+        <v>0.1566282</v>
+      </c>
+      <c r="P68">
+        <v>0.14972099999999999</v>
+      </c>
+      <c r="Q68">
+        <v>0.1218776</v>
+      </c>
+      <c r="R68">
+        <v>5.1503599999999997E-2</v>
+      </c>
+      <c r="S68">
+        <v>0.10913100000000001</v>
+      </c>
+      <c r="T68">
+        <v>9.39247E-2</v>
+      </c>
+      <c r="U68">
+        <v>9.95423E-2</v>
+      </c>
+      <c r="V68">
+        <v>0.1035594</v>
+      </c>
+      <c r="W68">
+        <v>5.7743900000000001E-2</v>
+      </c>
+      <c r="X68">
+        <v>6.05348E-2</v>
+      </c>
+      <c r="Y68">
+        <v>0.12821440000000001</v>
+      </c>
+      <c r="Z68">
+        <v>9.1439400000000004E-2</v>
+      </c>
+      <c r="AA68">
+        <v>7.2081999999999993E-2</v>
+      </c>
+      <c r="AB68">
+        <v>9.1803300000000004E-2</v>
+      </c>
+      <c r="AC68">
+        <v>8.8094599999999995E-2</v>
+      </c>
+      <c r="AD68">
+        <v>8.6147899999999999E-2</v>
+      </c>
+      <c r="AE68">
+        <v>9.5489900000000003E-2</v>
+      </c>
+      <c r="AF68">
+        <v>-5.9182000000000002E-3</v>
+      </c>
+      <c r="AG68">
+        <v>-3.8192E-3</v>
+      </c>
+      <c r="AH68">
+        <v>-2.5037000000000002E-3</v>
+      </c>
+      <c r="AI68">
+        <v>5.7850000000000002E-4</v>
+      </c>
+      <c r="AJ68">
+        <v>8.9817000000000004E-3</v>
+      </c>
+      <c r="AK68">
+        <v>4.4030000000000002E-4</v>
+      </c>
+      <c r="AL68">
+        <v>-3.2762999999999998E-3</v>
+      </c>
+      <c r="AM68">
+        <v>5.3447E-3</v>
+      </c>
+      <c r="AN68">
+        <v>6.1416600000000002E-2</v>
+      </c>
+      <c r="AO68">
+        <v>2.4001999999999999E-2</v>
+      </c>
+      <c r="AP68">
+        <v>2.5999E-3</v>
+      </c>
+      <c r="AQ68">
+        <v>-2.6505999999999999E-3</v>
+      </c>
+      <c r="AR68">
+        <v>2.2186500000000001E-2</v>
+      </c>
+      <c r="AS68">
+        <v>-1.64616E-2</v>
+      </c>
+      <c r="AT68">
+        <v>-1.51974E-2</v>
+      </c>
+      <c r="AU68">
+        <v>-8.0619000000000003E-3</v>
+      </c>
+      <c r="AV68">
+        <v>-4.7810699999999998E-2</v>
+      </c>
+      <c r="AW68">
+        <v>-1.29937E-2</v>
+      </c>
+      <c r="AX68">
+        <v>-4.1999000000000003E-3</v>
+      </c>
+      <c r="AY68">
+        <v>-8.0628000000000002E-3</v>
+      </c>
+      <c r="AZ68">
+        <v>-3.9616E-3</v>
+      </c>
+      <c r="BA68">
+        <v>-1.751E-4</v>
+      </c>
+      <c r="BB68">
+        <v>-4.8929999999999998E-3</v>
+      </c>
+      <c r="BC68">
+        <v>-4.6546000000000001E-3</v>
+      </c>
+      <c r="BD68">
+        <v>-6.4056E-3</v>
+      </c>
+      <c r="BE68">
+        <v>-4.4948000000000002E-3</v>
+      </c>
+      <c r="BF68">
+        <v>-4.8858E-3</v>
+      </c>
+      <c r="BG68">
+        <v>-5.6893999999999998E-3</v>
+      </c>
+      <c r="BH68">
+        <v>-8.9768000000000001E-3</v>
+      </c>
+      <c r="BI68">
+        <v>6.3020999999999997E-3</v>
+      </c>
+      <c r="BJ68">
+        <v>-4.4565399999999998E-2</v>
+      </c>
+      <c r="BK68">
+        <v>-0.16409399999999999</v>
+      </c>
+      <c r="BL68">
+        <v>-0.14949019999999999</v>
+      </c>
+      <c r="BM68">
+        <v>-6.4953399999999994E-2</v>
+      </c>
+      <c r="BN68">
+        <v>-0.15185209999999999</v>
+      </c>
+      <c r="BO68">
+        <v>-0.14156640000000001</v>
+      </c>
+      <c r="BP68">
+        <v>-2.6488000000000002E-3</v>
+      </c>
+      <c r="BQ68">
+        <v>-4.3956999999999998E-3</v>
+      </c>
+      <c r="BR68" t="s">
+        <v>76</v>
+      </c>
+      <c r="BS68">
+        <v>-2.9805999999999999E-3</v>
+      </c>
+      <c r="BT68">
+        <v>-4.5425100000000003E-2</v>
+      </c>
+      <c r="BU68">
+        <v>-3.8919999999999997E-4</v>
+      </c>
+      <c r="BV68">
+        <v>-2.1124299999999999E-2</v>
+      </c>
+      <c r="BW68">
+        <v>-2.5271600000000002E-2</v>
+      </c>
+      <c r="BX68">
+        <v>-3.2949100000000002E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>283</v>
+      </c>
+      <c r="C69" t="s">
+        <v>143</v>
+      </c>
+      <c r="D69">
+        <v>-7.1561000000000003E-3</v>
+      </c>
+      <c r="E69">
+        <v>-4.7565000000000003E-3</v>
+      </c>
+      <c r="F69">
+        <v>-5.9584E-3</v>
+      </c>
+      <c r="G69">
+        <v>3.4278299999999998E-2</v>
+      </c>
+      <c r="H69">
+        <v>-6.8830000000000002E-3</v>
+      </c>
+      <c r="I69">
+        <v>1.59515E-2</v>
+      </c>
+      <c r="J69">
+        <v>-4.0124999999999996E-3</v>
+      </c>
+      <c r="K69">
+        <v>3.7122299999999997E-2</v>
+      </c>
+      <c r="L69">
+        <v>-4.8479000000000001E-2</v>
+      </c>
+      <c r="M69">
+        <v>-1.9210999999999999E-2</v>
+      </c>
+      <c r="N69">
+        <v>-6.9490000000000003E-3</v>
+      </c>
+      <c r="O69">
+        <v>-1.17219E-2</v>
+      </c>
+      <c r="P69">
+        <v>-8.4063999999999996E-3</v>
+      </c>
+      <c r="Q69">
+        <v>1.6055E-2</v>
+      </c>
+      <c r="R69">
+        <v>3.2562300000000002E-2</v>
+      </c>
+      <c r="S69">
+        <v>2.21902E-2</v>
+      </c>
+      <c r="T69">
+        <v>2.8611500000000002E-2</v>
+      </c>
+      <c r="U69">
+        <v>2.56289E-2</v>
+      </c>
+      <c r="V69">
+        <v>2.6715099999999999E-2</v>
+      </c>
+      <c r="W69">
+        <v>7.3495000000000001E-3</v>
+      </c>
+      <c r="X69">
+        <v>2.9134899999999998E-2</v>
+      </c>
+      <c r="Y69">
+        <v>4.2407399999999998E-2</v>
+      </c>
+      <c r="Z69">
+        <v>4.5370099999999997E-2</v>
+      </c>
+      <c r="AA69">
+        <v>4.2508799999999999E-2</v>
+      </c>
+      <c r="AB69">
+        <v>3.87131E-2</v>
+      </c>
+      <c r="AC69">
+        <v>3.6703899999999998E-2</v>
+      </c>
+      <c r="AD69">
+        <v>3.9952700000000001E-2</v>
+      </c>
+      <c r="AE69">
+        <v>3.8029300000000002E-2</v>
+      </c>
+      <c r="AF69">
+        <v>3.09509E-2</v>
+      </c>
+      <c r="AG69">
+        <v>3.1742100000000002E-2</v>
+      </c>
+      <c r="AH69">
+        <v>3.37948E-2</v>
+      </c>
+      <c r="AI69">
+        <v>2.7879999999999999E-2</v>
+      </c>
+      <c r="AJ69">
+        <v>2.8461199999999999E-2</v>
+      </c>
+      <c r="AK69">
+        <v>3.5194000000000003E-2</v>
+      </c>
+      <c r="AL69">
+        <v>3.0195699999999999E-2</v>
+      </c>
+      <c r="AM69">
+        <v>2.6224500000000001E-2</v>
+      </c>
+      <c r="AN69">
+        <v>1.21945E-2</v>
+      </c>
+      <c r="AO69">
+        <v>2.8972600000000001E-2</v>
+      </c>
+      <c r="AP69">
+        <v>1.7764200000000001E-2</v>
+      </c>
+      <c r="AQ69">
+        <v>3.4165000000000001E-2</v>
+      </c>
+      <c r="AR69">
+        <v>1.35388E-2</v>
+      </c>
+      <c r="AS69">
+        <v>2.34246E-2</v>
+      </c>
+      <c r="AT69">
+        <v>2.8868399999999999E-2</v>
+      </c>
+      <c r="AU69">
+        <v>2.5782300000000001E-2</v>
+      </c>
+      <c r="AV69">
+        <v>3.9884999999999999E-3</v>
+      </c>
+      <c r="AW69">
+        <v>2.43804E-2</v>
+      </c>
+      <c r="AX69">
+        <v>2.7038900000000001E-2</v>
+      </c>
+      <c r="AY69">
+        <v>2.9104100000000001E-2</v>
+      </c>
+      <c r="AZ69">
+        <v>2.7902199999999999E-2</v>
+      </c>
+      <c r="BA69">
+        <v>2.13987E-2</v>
+      </c>
+      <c r="BB69">
+        <v>2.2140400000000001E-2</v>
+      </c>
+      <c r="BC69">
+        <v>2.7867200000000002E-2</v>
+      </c>
+      <c r="BD69">
+        <v>2.1825500000000001E-2</v>
+      </c>
+      <c r="BE69">
+        <v>2.2368900000000001E-2</v>
+      </c>
+      <c r="BF69">
+        <v>2.63374E-2</v>
+      </c>
+      <c r="BG69">
+        <v>3.0160699999999999E-2</v>
+      </c>
+      <c r="BH69">
+        <v>1.84087E-2</v>
+      </c>
+      <c r="BI69">
+        <v>1.91208E-2</v>
+      </c>
+      <c r="BJ69">
+        <v>6.8168599999999996E-2</v>
+      </c>
+      <c r="BK69">
+        <v>7.1095099999999994E-2</v>
+      </c>
+      <c r="BL69">
+        <v>7.7735399999999996E-2</v>
+      </c>
+      <c r="BM69">
+        <v>9.34059E-2</v>
+      </c>
+      <c r="BN69">
+        <v>8.3501000000000006E-2</v>
+      </c>
+      <c r="BO69">
+        <v>7.2125999999999996E-2</v>
+      </c>
+      <c r="BP69">
+        <v>3.3177499999999999E-2</v>
+      </c>
+      <c r="BQ69">
+        <v>4.3974800000000001E-2</v>
+      </c>
+      <c r="BR69">
+        <v>-5.9929999999999998E-4</v>
+      </c>
+      <c r="BS69" t="s">
+        <v>76</v>
+      </c>
+      <c r="BT69">
+        <v>3.18412E-2</v>
+      </c>
+      <c r="BU69">
+        <v>4.91954E-2</v>
+      </c>
+      <c r="BV69">
+        <v>8.9087200000000005E-2</v>
+      </c>
+      <c r="BW69">
+        <v>0.1162301</v>
+      </c>
+      <c r="BX69">
+        <v>9.2856300000000003E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>1848</v>
+      </c>
+      <c r="B70" t="s">
+        <v>159</v>
+      </c>
+      <c r="C70" t="s">
+        <v>144</v>
+      </c>
+      <c r="D70">
+        <v>1.0483000000000001E-3</v>
+      </c>
+      <c r="E70">
+        <v>3.0279999999999999E-4</v>
+      </c>
+      <c r="F70">
+        <v>-1.4629000000000001E-3</v>
+      </c>
+      <c r="G70">
+        <v>6.3429399999999997E-2</v>
+      </c>
+      <c r="H70">
+        <v>-5.9630000000000002E-4</v>
+      </c>
+      <c r="I70">
+        <v>-6.4238100000000006E-2</v>
+      </c>
+      <c r="J70">
+        <v>1.5603000000000001E-2</v>
+      </c>
+      <c r="K70">
+        <v>1.2632300000000001E-2</v>
+      </c>
+      <c r="L70">
+        <v>-6.5944000000000003E-3</v>
+      </c>
+      <c r="M70">
+        <v>4.4711000000000001E-2</v>
+      </c>
+      <c r="N70">
+        <v>9.4030699999999995E-2</v>
+      </c>
+      <c r="O70">
+        <v>0.1194215</v>
+      </c>
+      <c r="P70">
+        <v>0.1021445</v>
+      </c>
+      <c r="Q70">
+        <v>9.2569000000000002E-3</v>
+      </c>
+      <c r="R70">
+        <v>0.1046864</v>
+      </c>
+      <c r="S70">
+        <v>5.2614300000000003E-2</v>
+      </c>
+      <c r="T70">
+        <v>4.77905E-2</v>
+      </c>
+      <c r="U70">
+        <v>5.9605100000000001E-2</v>
+      </c>
+      <c r="V70">
+        <v>6.9029699999999999E-2</v>
+      </c>
+      <c r="W70">
+        <v>-1.4881999999999999E-2</v>
+      </c>
+      <c r="X70">
+        <v>3.1045000000000001E-3</v>
+      </c>
+      <c r="Y70">
+        <v>-4.0988299999999998E-2</v>
+      </c>
+      <c r="Z70">
+        <v>-1.4855999999999999E-2</v>
+      </c>
+      <c r="AA70">
+        <v>-2.33878E-2</v>
+      </c>
+      <c r="AB70">
+        <v>-1.7691599999999998E-2</v>
+      </c>
+      <c r="AC70">
+        <v>-1.41219E-2</v>
+      </c>
+      <c r="AD70">
+        <v>-2.2124399999999999E-2</v>
+      </c>
+      <c r="AE70">
+        <v>-2.5379800000000001E-2</v>
+      </c>
+      <c r="AF70">
+        <v>2.32879E-2</v>
+      </c>
+      <c r="AG70">
+        <v>1.0635E-2</v>
+      </c>
+      <c r="AH70">
+        <v>1.04303E-2</v>
+      </c>
+      <c r="AI70">
+        <v>1.4507900000000001E-2</v>
+      </c>
+      <c r="AJ70">
+        <v>9.4351999999999995E-3</v>
+      </c>
+      <c r="AK70">
+        <v>-2.9324699999999999E-2</v>
+      </c>
+      <c r="AL70">
+        <v>-9.0129999999999995E-4</v>
+      </c>
+      <c r="AM70">
+        <v>2.6459900000000001E-2</v>
+      </c>
+      <c r="AN70">
+        <v>6.1288200000000001E-2</v>
+      </c>
+      <c r="AO70">
+        <v>6.4654500000000004E-2</v>
+      </c>
+      <c r="AP70">
+        <v>-7.1542999999999997E-3</v>
+      </c>
+      <c r="AQ70">
+        <v>-2.6586000000000001E-3</v>
+      </c>
+      <c r="AR70">
+        <v>1.52753E-2</v>
+      </c>
+      <c r="AS70">
+        <v>-4.8393999999999998E-3</v>
+      </c>
+      <c r="AT70">
+        <v>6.0077999999999998E-3</v>
+      </c>
+      <c r="AU70">
+        <v>2.7820000000000002E-3</v>
+      </c>
+      <c r="AV70">
+        <v>-4.1916500000000002E-2</v>
+      </c>
+      <c r="AW70">
+        <v>-6.4625999999999998E-3</v>
+      </c>
+      <c r="AX70">
+        <v>4.5595999999999996E-3</v>
+      </c>
+      <c r="AY70">
+        <v>6.9670000000000001E-3</v>
+      </c>
+      <c r="AZ70">
+        <v>-4.7137999999999998E-3</v>
+      </c>
+      <c r="BA70">
+        <v>2.1797000000000001E-3</v>
+      </c>
+      <c r="BB70">
+        <v>1.5162399999999999E-2</v>
+      </c>
+      <c r="BC70">
+        <v>6.4559999999999997E-4</v>
+      </c>
+      <c r="BD70">
+        <v>1.5280800000000001E-2</v>
+      </c>
+      <c r="BE70">
+        <v>1.6865399999999999E-2</v>
+      </c>
+      <c r="BF70">
+        <v>-2.085E-4</v>
+      </c>
+      <c r="BG70">
+        <v>9.0439999999999997E-4</v>
+      </c>
+      <c r="BH70">
+        <v>-1.3344E-2</v>
+      </c>
+      <c r="BI70">
+        <v>5.8001400000000002E-2</v>
+      </c>
+      <c r="BJ70">
+        <v>2.60606E-2</v>
+      </c>
+      <c r="BK70">
+        <v>-5.3664000000000003E-2</v>
+      </c>
+      <c r="BL70">
+        <v>-9.2262000000000004E-3</v>
+      </c>
+      <c r="BM70">
+        <v>-2.2770499999999999E-2</v>
+      </c>
+      <c r="BN70">
+        <v>-3.2540600000000003E-2</v>
+      </c>
+      <c r="BO70">
+        <v>-1.9518999999999999E-3</v>
+      </c>
+      <c r="BP70">
+        <v>2.08858E-2</v>
+      </c>
+      <c r="BQ70">
+        <v>3.1670999999999998E-2</v>
+      </c>
+      <c r="BR70">
+        <v>-8.6745999999999993E-3</v>
+      </c>
+      <c r="BS70">
+        <v>4.4508300000000001E-2</v>
+      </c>
+      <c r="BT70" t="s">
+        <v>76</v>
+      </c>
+      <c r="BU70">
+        <v>2.8103199999999998E-2</v>
+      </c>
+      <c r="BV70">
+        <v>0.25444919999999999</v>
+      </c>
+      <c r="BW70">
+        <v>0.1599468</v>
+      </c>
+      <c r="BX70">
+        <v>6.7256300000000005E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>682</v>
+      </c>
+      <c r="B71" t="s">
+        <v>159</v>
+      </c>
+      <c r="C71" t="s">
+        <v>145</v>
+      </c>
+      <c r="D71">
+        <v>-7.2521E-3</v>
+      </c>
+      <c r="E71">
+        <v>-5.9947000000000004E-3</v>
+      </c>
+      <c r="F71">
+        <v>-5.6579999999999998E-3</v>
+      </c>
+      <c r="G71">
+        <v>9.4608000000000001E-3</v>
+      </c>
+      <c r="H71">
+        <v>-6.1865000000000002E-3</v>
+      </c>
+      <c r="I71">
+        <v>-4.5970000000000004E-3</v>
+      </c>
+      <c r="J71">
+        <v>-4.9953000000000003E-3</v>
+      </c>
+      <c r="K71">
+        <v>2.6625599999999999E-2</v>
+      </c>
+      <c r="L71">
+        <v>-1.7845300000000001E-2</v>
+      </c>
+      <c r="M71">
+        <v>-1.1697000000000001E-3</v>
+      </c>
+      <c r="N71">
+        <v>3.5539999999999999E-3</v>
+      </c>
+      <c r="O71">
+        <v>4.8298999999999998E-3</v>
+      </c>
+      <c r="P71">
+        <v>8.2803000000000009E-3</v>
+      </c>
+      <c r="Q71">
+        <v>2.2490400000000001E-2</v>
+      </c>
+      <c r="R71">
+        <v>2.1550300000000001E-2</v>
+      </c>
+      <c r="S71">
+        <v>2.85002E-2</v>
+      </c>
+      <c r="T71">
+        <v>2.6760300000000001E-2</v>
+      </c>
+      <c r="U71">
+        <v>2.9464000000000001E-2</v>
+      </c>
+      <c r="V71">
+        <v>2.50599E-2</v>
+      </c>
+      <c r="W71">
+        <v>2.7218599999999999E-2</v>
+      </c>
+      <c r="X71">
+        <v>3.13038E-2</v>
+      </c>
+      <c r="Y71">
+        <v>2.77711E-2</v>
+      </c>
+      <c r="Z71">
+        <v>2.6134999999999999E-2</v>
+      </c>
+      <c r="AA71">
+        <v>3.05268E-2</v>
+      </c>
+      <c r="AB71">
+        <v>3.2097300000000002E-2</v>
+      </c>
+      <c r="AC71">
+        <v>1.7262199999999998E-2</v>
+      </c>
+      <c r="AD71">
+        <v>2.2057799999999999E-2</v>
+      </c>
+      <c r="AE71">
+        <v>2.4018399999999999E-2</v>
+      </c>
+      <c r="AF71">
+        <v>3.8567700000000003E-2</v>
+      </c>
+      <c r="AG71">
+        <v>3.8164099999999999E-2</v>
+      </c>
+      <c r="AH71">
+        <v>4.6556500000000001E-2</v>
+      </c>
+      <c r="AI71">
+        <v>4.0509299999999998E-2</v>
+      </c>
+      <c r="AJ71">
+        <v>3.6329399999999998E-2</v>
+      </c>
+      <c r="AK71">
+        <v>1.6767000000000001E-2</v>
+      </c>
+      <c r="AL71">
+        <v>3.5091400000000002E-2</v>
+      </c>
+      <c r="AM71">
+        <v>3.6419800000000002E-2</v>
+      </c>
+      <c r="AN71">
+        <v>3.1416E-3</v>
+      </c>
+      <c r="AO71">
+        <v>1.8098400000000001E-2</v>
+      </c>
+      <c r="AP71">
+        <v>2.1635100000000001E-2</v>
+      </c>
+      <c r="AQ71">
+        <v>3.9829299999999998E-2</v>
+      </c>
+      <c r="AR71">
+        <v>3.0866000000000001E-2</v>
+      </c>
+      <c r="AS71">
+        <v>3.09188E-2</v>
+      </c>
+      <c r="AT71">
+        <v>2.7898800000000001E-2</v>
+      </c>
+      <c r="AU71">
+        <v>3.04566E-2</v>
+      </c>
+      <c r="AV71">
+        <v>1.2653899999999999E-2</v>
+      </c>
+      <c r="AW71">
+        <v>2.9549300000000001E-2</v>
+      </c>
+      <c r="AX71">
+        <v>2.4475799999999999E-2</v>
+      </c>
+      <c r="AY71">
+        <v>3.4078400000000002E-2</v>
+      </c>
+      <c r="AZ71">
+        <v>3.54014E-2</v>
+      </c>
+      <c r="BA71">
+        <v>7.9325999999999997E-3</v>
+      </c>
+      <c r="BB71">
+        <v>3.42955E-2</v>
+      </c>
+      <c r="BC71">
+        <v>3.68548E-2</v>
+      </c>
+      <c r="BD71">
+        <v>3.5120499999999999E-2</v>
+      </c>
+      <c r="BE71">
+        <v>3.9272899999999999E-2</v>
+      </c>
+      <c r="BF71">
+        <v>4.1415100000000003E-2</v>
+      </c>
+      <c r="BG71">
+        <v>4.2076299999999997E-2</v>
+      </c>
+      <c r="BH71">
+        <v>2.5755900000000002E-2</v>
+      </c>
+      <c r="BI71">
+        <v>3.52349E-2</v>
+      </c>
+      <c r="BJ71">
+        <v>-1.8487699999999999E-2</v>
+      </c>
+      <c r="BK71">
+        <v>4.7630400000000003E-2</v>
+      </c>
+      <c r="BL71">
+        <v>2.0623800000000001E-2</v>
+      </c>
+      <c r="BM71">
+        <v>3.9510999999999998E-2</v>
+      </c>
+      <c r="BN71">
+        <v>1.4223100000000001E-2</v>
+      </c>
+      <c r="BO71">
+        <v>2.17953E-2</v>
+      </c>
+      <c r="BP71">
+        <v>3.2727699999999998E-2</v>
+      </c>
+      <c r="BQ71">
+        <v>2.9859199999999999E-2</v>
+      </c>
+      <c r="BR71">
+        <v>-5.4222000000000003E-3</v>
+      </c>
+      <c r="BS71">
+        <v>3.1565700000000002E-2</v>
+      </c>
+      <c r="BT71">
+        <v>5.7778400000000001E-2</v>
+      </c>
+      <c r="BU71" t="s">
+        <v>76</v>
+      </c>
+      <c r="BV71">
+        <v>2.3107699999999998E-2</v>
+      </c>
+      <c r="BW71">
+        <v>3.5760300000000002E-2</v>
+      </c>
+      <c r="BX71">
+        <v>4.8668299999999998E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>1357</v>
+      </c>
+      <c r="B72" t="s">
+        <v>159</v>
+      </c>
+      <c r="C72" t="s">
+        <v>146</v>
+      </c>
+      <c r="D72">
+        <v>6.2021000000000003E-3</v>
+      </c>
+      <c r="E72">
+        <v>-1.5969000000000001E-3</v>
+      </c>
+      <c r="F72">
+        <v>-5.8542000000000004E-3</v>
+      </c>
+      <c r="G72">
+        <v>6.5760299999999994E-2</v>
+      </c>
+      <c r="H72">
+        <v>-5.7128999999999999E-3</v>
+      </c>
+      <c r="I72">
+        <v>-1.1170899999999999E-2</v>
+      </c>
+      <c r="J72">
+        <v>1.5773E-3</v>
+      </c>
+      <c r="K72">
+        <v>0.10361339999999999</v>
+      </c>
+      <c r="L72">
+        <v>-1.2283199999999999E-2</v>
+      </c>
+      <c r="M72">
+        <v>1.2415499999999999E-2</v>
+      </c>
+      <c r="N72">
+        <v>3.6344300000000003E-2</v>
+      </c>
+      <c r="O72">
+        <v>2.5785800000000001E-2</v>
+      </c>
+      <c r="P72">
+        <v>3.3962899999999997E-2</v>
+      </c>
+      <c r="Q72">
+        <v>3.3222399999999999E-2</v>
+      </c>
+      <c r="R72">
+        <v>-5.1317000000000003E-3</v>
+      </c>
+      <c r="S72">
+        <v>3.9946599999999999E-2</v>
+      </c>
+      <c r="T72">
+        <v>-5.4502999999999999E-3</v>
+      </c>
+      <c r="U72">
+        <v>3.2836200000000003E-2</v>
+      </c>
+      <c r="V72">
+        <v>2.2251300000000002E-2</v>
+      </c>
+      <c r="W72">
+        <v>0.100746</v>
+      </c>
+      <c r="X72">
+        <v>7.9295299999999999E-2</v>
+      </c>
+      <c r="Y72">
+        <v>5.5151899999999997E-2</v>
+      </c>
+      <c r="Z72">
+        <v>2.1770500000000002E-2</v>
+      </c>
+      <c r="AA72">
+        <v>6.7644000000000003E-3</v>
+      </c>
+      <c r="AB72">
+        <v>1.15599E-2</v>
+      </c>
+      <c r="AC72">
+        <v>3.13079E-2</v>
+      </c>
+      <c r="AD72">
+        <v>1.7551500000000001E-2</v>
+      </c>
+      <c r="AE72">
+        <v>1.25354E-2</v>
+      </c>
+      <c r="AF72">
+        <v>8.8830000000000003E-3</v>
+      </c>
+      <c r="AG72">
+        <v>4.7669000000000001E-3</v>
+      </c>
+      <c r="AH72">
+        <v>4.793E-4</v>
+      </c>
+      <c r="AI72">
+        <v>1.14625E-2</v>
+      </c>
+      <c r="AJ72">
+        <v>2.7111000000000001E-3</v>
+      </c>
+      <c r="AK72">
+        <v>-1.57606E-2</v>
+      </c>
+      <c r="AL72">
+        <v>4.5019999999999999E-3</v>
+      </c>
+      <c r="AM72">
+        <v>1.9751299999999999E-2</v>
+      </c>
+      <c r="AN72">
+        <v>-3.9321099999999998E-2</v>
+      </c>
+      <c r="AO72">
+        <v>-1.0195900000000001E-2</v>
+      </c>
+      <c r="AP72">
+        <v>2.4754700000000001E-2</v>
+      </c>
+      <c r="AQ72">
+        <v>3.4764000000000001E-3</v>
+      </c>
+      <c r="AR72">
+        <v>1.6969999999999999E-3</v>
+      </c>
+      <c r="AS72">
+        <v>-3.7409999999999999E-4</v>
+      </c>
+      <c r="AT72">
+        <v>-1.24954E-2</v>
+      </c>
+      <c r="AU72">
+        <v>-2.7550999999999999E-3</v>
+      </c>
+      <c r="AV72">
+        <v>-7.2858400000000004E-2</v>
+      </c>
+      <c r="AW72">
+        <v>-4.7685999999999996E-3</v>
+      </c>
+      <c r="AX72">
+        <v>-1.14968E-2</v>
+      </c>
+      <c r="AY72">
+        <v>5.2399999999999999E-3</v>
+      </c>
+      <c r="AZ72">
+        <v>-1.3156000000000001E-3</v>
+      </c>
+      <c r="BA72">
+        <v>-2.65069E-2</v>
+      </c>
+      <c r="BB72">
+        <v>4.8441600000000001E-2</v>
+      </c>
+      <c r="BC72">
+        <v>1.10908E-2</v>
+      </c>
+      <c r="BD72">
+        <v>4.7636699999999997E-2</v>
+      </c>
+      <c r="BE72">
+        <v>5.2246899999999999E-2</v>
+      </c>
+      <c r="BF72">
+        <v>2.3132000000000001E-3</v>
+      </c>
+      <c r="BG72">
+        <v>4.1862000000000002E-3</v>
+      </c>
+      <c r="BH72">
+        <v>-6.0280399999999998E-2</v>
+      </c>
+      <c r="BI72">
+        <v>1.4261899999999999E-2</v>
+      </c>
+      <c r="BJ72">
+        <v>1.34939E-2</v>
+      </c>
+      <c r="BK72">
+        <v>-5.7390799999999999E-2</v>
+      </c>
+      <c r="BL72">
+        <v>-6.2704099999999999E-2</v>
+      </c>
+      <c r="BM72">
+        <v>-4.4412E-2</v>
+      </c>
+      <c r="BN72">
+        <v>-4.0852300000000001E-2</v>
+      </c>
+      <c r="BO72">
+        <v>-3.1779700000000001E-2</v>
+      </c>
+      <c r="BP72">
+        <v>1.5514E-2</v>
+      </c>
+      <c r="BQ72">
+        <v>2.02337E-2</v>
+      </c>
+      <c r="BR72">
+        <v>2.55009E-2</v>
+      </c>
+      <c r="BS72">
+        <v>5.39052E-2</v>
+      </c>
+      <c r="BT72">
+        <v>0.17330999999999999</v>
+      </c>
+      <c r="BU72">
+        <v>1.6572699999999999E-2</v>
+      </c>
+      <c r="BV72" t="s">
+        <v>76</v>
+      </c>
+      <c r="BW72">
+        <v>0.14723720000000001</v>
+      </c>
+      <c r="BX72">
+        <v>4.9982699999999998E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>769</v>
+      </c>
+      <c r="B73" t="s">
+        <v>159</v>
+      </c>
+      <c r="C73" t="s">
+        <v>147</v>
+      </c>
+      <c r="D73">
+        <v>5.2349999999999999E-4</v>
+      </c>
+      <c r="E73">
+        <v>-3.5403000000000001E-3</v>
+      </c>
+      <c r="F73">
+        <v>-2.7440300000000001E-2</v>
+      </c>
+      <c r="G73">
+        <v>-4.88578E-2</v>
+      </c>
+      <c r="H73">
+        <v>-4.8278000000000001E-3</v>
+      </c>
+      <c r="I73">
+        <v>0.13069610000000001</v>
+      </c>
+      <c r="J73">
+        <v>-3.5056000000000002E-3</v>
+      </c>
+      <c r="K73">
+        <v>4.9656699999999998E-2</v>
+      </c>
+      <c r="L73">
+        <v>-0.14616199999999999</v>
+      </c>
+      <c r="M73">
+        <v>8.5356799999999997E-2</v>
+      </c>
+      <c r="N73">
+        <v>1.9044100000000001E-2</v>
+      </c>
+      <c r="O73">
+        <v>5.18664E-2</v>
+      </c>
+      <c r="P73">
+        <v>5.4780000000000002E-2</v>
+      </c>
+      <c r="Q73">
+        <v>3.21631E-2</v>
+      </c>
+      <c r="R73">
+        <v>5.0844800000000002E-2</v>
+      </c>
+      <c r="S73">
+        <v>3.5750799999999999E-2</v>
+      </c>
+      <c r="T73">
+        <v>-1.32161E-2</v>
+      </c>
+      <c r="U73">
+        <v>2.0242400000000001E-2</v>
+      </c>
+      <c r="V73">
+        <v>1.10229E-2</v>
+      </c>
+      <c r="W73">
+        <v>1.45661E-2</v>
+      </c>
+      <c r="X73">
+        <v>8.8363000000000001E-3</v>
+      </c>
+      <c r="Y73">
+        <v>1.8705699999999999E-2</v>
+      </c>
+      <c r="Z73">
+        <v>1.2549E-3</v>
+      </c>
+      <c r="AA73">
+        <v>-3.60568E-2</v>
+      </c>
+      <c r="AB73">
+        <v>-1.7895999999999999E-2</v>
+      </c>
+      <c r="AC73">
+        <v>-9.2041999999999992E-3</v>
+      </c>
+      <c r="AD73">
+        <v>-4.1347299999999997E-2</v>
+      </c>
+      <c r="AE73">
+        <v>-1.37786E-2</v>
+      </c>
+      <c r="AF73">
+        <v>-8.6420000000000004E-3</v>
+      </c>
+      <c r="AG73">
+        <v>-1.7875599999999998E-2</v>
+      </c>
+      <c r="AH73">
+        <v>-3.5084000000000001E-3</v>
+      </c>
+      <c r="AI73">
+        <v>1.6877900000000001E-2</v>
+      </c>
+      <c r="AJ73">
+        <v>4.4364000000000001E-3</v>
+      </c>
+      <c r="AK73">
+        <v>-2.86895E-2</v>
+      </c>
+      <c r="AL73">
+        <v>4.8507999999999997E-3</v>
+      </c>
+      <c r="AM73">
+        <v>9.5560000000000003E-4</v>
+      </c>
+      <c r="AN73">
+        <v>-2.4782499999999999E-2</v>
+      </c>
+      <c r="AO73">
+        <v>-7.1154E-3</v>
+      </c>
+      <c r="AP73">
+        <v>7.2979999999999996E-4</v>
+      </c>
+      <c r="AQ73">
+        <v>9.8647000000000006E-3</v>
+      </c>
+      <c r="AR73">
+        <v>-1.6638500000000001E-2</v>
+      </c>
+      <c r="AS73">
+        <v>-1.36883E-2</v>
+      </c>
+      <c r="AT73">
+        <v>-3.4221799999999997E-2</v>
+      </c>
+      <c r="AU73">
+        <v>-4.5206000000000003E-2</v>
+      </c>
+      <c r="AV73">
+        <v>-7.1963399999999997E-2</v>
+      </c>
+      <c r="AW73">
+        <v>-2.5054199999999999E-2</v>
+      </c>
+      <c r="AX73">
+        <v>-7.29683E-2</v>
+      </c>
+      <c r="AY73">
+        <v>-1.4532700000000001E-2</v>
+      </c>
+      <c r="AZ73">
+        <v>2.332E-4</v>
+      </c>
+      <c r="BA73">
+        <v>-2.5141299999999998E-2</v>
+      </c>
+      <c r="BB73">
+        <v>4.3973999999999999E-2</v>
+      </c>
+      <c r="BC73">
+        <v>1.6671100000000001E-2</v>
+      </c>
+      <c r="BD73">
+        <v>5.1164599999999998E-2</v>
+      </c>
+      <c r="BE73">
+        <v>4.4607599999999997E-2</v>
+      </c>
+      <c r="BF73">
+        <v>8.7112999999999999E-3</v>
+      </c>
+      <c r="BG73">
+        <v>8.4457000000000004E-3</v>
+      </c>
+      <c r="BH73">
+        <v>0.1086217</v>
+      </c>
+      <c r="BI73">
+        <v>1.38526E-2</v>
+      </c>
+      <c r="BJ73">
+        <v>9.4002299999999997E-2</v>
+      </c>
+      <c r="BK73">
+        <v>2.0753199999999999E-2</v>
+      </c>
+      <c r="BL73">
+        <v>3.8139899999999997E-2</v>
+      </c>
+      <c r="BM73">
+        <v>3.5591600000000001E-2</v>
+      </c>
+      <c r="BN73">
+        <v>2.48203E-2</v>
+      </c>
+      <c r="BO73">
+        <v>3.2276600000000003E-2</v>
+      </c>
+      <c r="BP73">
+        <v>9.4245000000000006E-3</v>
+      </c>
+      <c r="BQ73">
+        <v>1.6187699999999999E-2</v>
+      </c>
+      <c r="BR73">
+        <v>3.1831400000000003E-2</v>
+      </c>
+      <c r="BS73">
+        <v>7.7706600000000001E-2</v>
+      </c>
+      <c r="BT73">
+        <v>-3.4128800000000001E-2</v>
+      </c>
+      <c r="BU73">
+        <v>2.1271100000000001E-2</v>
+      </c>
+      <c r="BV73">
+        <v>1.8807500000000001E-2</v>
+      </c>
+      <c r="BW73" t="s">
+        <v>76</v>
+      </c>
+      <c r="BX73">
+        <v>-9.5649999999999999E-4</v>
+      </c>
+    </row>
+    <row r="74" spans="1:76" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>1141</v>
+      </c>
+      <c r="B74" t="s">
+        <v>159</v>
+      </c>
+      <c r="C74" t="s">
+        <v>148</v>
+      </c>
+      <c r="D74">
+        <v>-4.9468000000000003E-3</v>
+      </c>
+      <c r="E74">
+        <v>-3.5948E-3</v>
+      </c>
+      <c r="F74">
+        <v>-1.2750900000000001E-2</v>
+      </c>
+      <c r="G74">
+        <v>5.4566900000000002E-2</v>
+      </c>
+      <c r="H74">
+        <v>-7.6001000000000003E-3</v>
+      </c>
+      <c r="I74">
+        <v>2.9268300000000001E-2</v>
+      </c>
+      <c r="J74">
+        <v>-2.6242000000000001E-3</v>
+      </c>
+      <c r="K74">
+        <v>8.9881900000000001E-2</v>
+      </c>
+      <c r="L74">
+        <v>-1.4209400000000001E-2</v>
+      </c>
+      <c r="M74">
+        <v>5.6994000000000003E-2</v>
+      </c>
+      <c r="N74">
+        <v>6.6618999999999998E-2</v>
+      </c>
+      <c r="O74">
+        <v>7.7400399999999994E-2</v>
+      </c>
+      <c r="P74">
+        <v>4.3133400000000002E-2</v>
+      </c>
+      <c r="Q74">
+        <v>9.7681599999999993E-2</v>
+      </c>
+      <c r="R74">
+        <v>6.6967799999999994E-2</v>
+      </c>
+      <c r="S74">
+        <v>0.1200681</v>
+      </c>
+      <c r="T74">
+        <v>9.7840499999999997E-2</v>
+      </c>
+      <c r="U74">
+        <v>9.4077300000000003E-2</v>
+      </c>
+      <c r="V74">
+        <v>9.2658099999999993E-2</v>
+      </c>
+      <c r="W74">
+        <v>9.0069499999999997E-2</v>
+      </c>
+      <c r="X74">
+        <v>0.1135896</v>
+      </c>
+      <c r="Y74">
+        <v>0.10667260000000001</v>
+      </c>
+      <c r="Z74">
+        <v>7.7293899999999999E-2</v>
+      </c>
+      <c r="AA74">
+        <v>5.6167300000000003E-2</v>
+      </c>
+      <c r="AB74">
+        <v>5.66802E-2</v>
+      </c>
+      <c r="AC74">
+        <v>4.8408199999999998E-2</v>
+      </c>
+      <c r="AD74">
+        <v>2.8824200000000001E-2</v>
+      </c>
+      <c r="AE74">
+        <v>5.6967999999999998E-2</v>
+      </c>
+      <c r="AF74">
+        <v>2.2813E-3</v>
+      </c>
+      <c r="AG74">
+        <v>8.9059999999999996E-4</v>
+      </c>
+      <c r="AH74">
+        <v>-1.574E-4</v>
+      </c>
+      <c r="AI74">
+        <v>3.9221000000000004E-3</v>
+      </c>
+      <c r="AJ74">
+        <v>-1.38858E-2</v>
+      </c>
+      <c r="AK74">
+        <v>-6.7521999999999999E-3</v>
+      </c>
+      <c r="AL74">
+        <v>7.2804000000000002E-3</v>
+      </c>
+      <c r="AM74">
+        <v>7.8869000000000005E-3</v>
+      </c>
+      <c r="AN74">
+        <v>2.7861000000000001E-3</v>
+      </c>
+      <c r="AO74">
+        <v>-1.5076E-3</v>
+      </c>
+      <c r="AP74">
+        <v>1.4900999999999999E-2</v>
+      </c>
+      <c r="AQ74">
+        <v>9.2197000000000008E-3</v>
+      </c>
+      <c r="AR74">
+        <v>-8.7530999999999998E-3</v>
+      </c>
+      <c r="AS74">
+        <v>1.5721200000000001E-2</v>
+      </c>
+      <c r="AT74">
+        <v>-1.1918099999999999E-2</v>
+      </c>
+      <c r="AU74">
+        <v>1.2652800000000001E-2</v>
+      </c>
+      <c r="AV74">
+        <v>-1.05968E-2</v>
+      </c>
+      <c r="AW74">
+        <v>1.1032399999999999E-2</v>
+      </c>
+      <c r="AX74">
+        <v>7.6524999999999996E-3</v>
+      </c>
+      <c r="AY74">
+        <v>1.9103E-3</v>
+      </c>
+      <c r="AZ74">
+        <v>1.2335E-2</v>
+      </c>
+      <c r="BA74">
+        <v>-5.0508999999999997E-3</v>
+      </c>
+      <c r="BB74">
+        <v>1.4376E-3</v>
+      </c>
+      <c r="BC74">
+        <v>1.7613799999999999E-2</v>
+      </c>
+      <c r="BD74">
+        <v>2.2577000000000001E-3</v>
+      </c>
+      <c r="BE74">
+        <v>3.6091000000000001E-3</v>
+      </c>
+      <c r="BF74">
+        <v>8.796E-3</v>
+      </c>
+      <c r="BG74">
+        <v>2.8744999999999999E-3</v>
+      </c>
+      <c r="BH74">
+        <v>3.5382799999999999E-2</v>
+      </c>
+      <c r="BI74">
+        <v>1.0943400000000001E-2</v>
+      </c>
+      <c r="BJ74">
+        <v>7.2981199999999996E-2</v>
+      </c>
+      <c r="BK74">
+        <v>6.10167E-2</v>
+      </c>
+      <c r="BL74">
+        <v>7.1942800000000001E-2</v>
+      </c>
+      <c r="BM74">
+        <v>5.0375900000000001E-2</v>
+      </c>
+      <c r="BN74">
+        <v>7.0275500000000005E-2</v>
+      </c>
+      <c r="BO74">
+        <v>3.9641299999999997E-2</v>
+      </c>
+      <c r="BP74">
+        <v>1.9149200000000002E-2</v>
+      </c>
+      <c r="BQ74">
+        <v>1.5849599999999998E-2</v>
+      </c>
+      <c r="BR74">
+        <v>2.2957600000000002E-2</v>
+      </c>
+      <c r="BS74">
+        <v>8.4461099999999997E-2</v>
+      </c>
+      <c r="BT74">
+        <v>6.22792E-2</v>
+      </c>
+      <c r="BU74">
+        <v>2.1286099999999999E-2</v>
+      </c>
+      <c r="BV74">
+        <v>9.6969399999999997E-2</v>
+      </c>
+      <c r="BW74">
+        <v>0.184307</v>
+      </c>
+      <c r="BX74" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:BQ67">
+  <conditionalFormatting sqref="B11:B14">
     <cfRule type="colorScale" priority="7">
       <colorScale>
-        <cfvo type="num" val="-0.5"/>
+        <cfvo type="num" val="-0.3"/>
         <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.5"/>
-        <color rgb="FFFF0000"/>
-        <color theme="0"/>
-        <color rgb="FF00B050"/>
+        <cfvo type="num" val="0.3"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B11:B14">
+  <conditionalFormatting sqref="B21:B24">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="-0.3"/>
@@ -15241,7 +18297,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B21:B24">
+  <conditionalFormatting sqref="B26:B29">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="num" val="-0.3"/>
@@ -15253,7 +18309,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B26:B29">
+  <conditionalFormatting sqref="B43:B48">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="num" val="-0.3"/>
@@ -15265,7 +18321,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B43:B48">
+  <conditionalFormatting sqref="B53:B57">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="num" val="-0.3"/>
@@ -15277,7 +18333,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B53:B57">
+  <conditionalFormatting sqref="B58:B59">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="-0.3"/>
@@ -15289,12 +18345,12 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B58:B59">
+  <conditionalFormatting sqref="D2:BX74">
     <cfRule type="colorScale" priority="1">
       <colorScale>
-        <cfvo type="num" val="-0.3"/>
+        <cfvo type="num" val="-0.5"/>
         <cfvo type="num" val="0"/>
-        <cfvo type="num" val="0.3"/>
+        <cfvo type="num" val="0.5"/>
         <color rgb="FFF8696B"/>
         <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>

</xml_diff>